<commit_message>
update spreadsheet & rerun scripts
</commit_message>
<xml_diff>
--- a/02-data/03-final-RA.xlsx
+++ b/02-data/03-final-RA.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="906" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1053" uniqueCount="572">
   <si>
     <t>framework_id</t>
   </si>
@@ -1388,6 +1388,9 @@
     <t xml:space="preserve">visualization by TensorBoard. </t>
   </si>
   <si>
+    <t>TensorBoard</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <color rgb="FF1155CC"/>
@@ -2717,9 +2720,6 @@
 def plot_results/ plot_curves</t>
   </si>
   <si>
-    <t>TensorBoard</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://github.com/DLR-RM/rl-baselines3-zoo/blob/master/rl_zoo3/train.py  </t>
   </si>
   <si>
@@ -2957,6 +2957,39 @@
   </si>
   <si>
     <t>manage RLlib experiments through an instance of the Algorithm class, share class with Framework Orchestrator, mix responsibilities</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/ray-project/ray/blob/master/python/ray/tune/tuner.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>class Tuner:
+    """Tuner is the recommended way of launching hyperparameter tuning jobs with Ray Tune.
+tune.Tuner(
+    config.algo_class,
+    param_space=config,
+    # Specify a stopping criterion. Note that the criterion has to match one of the
+    # pretty printed result metrics from the results returned previously by
+    # ``.train()``. Also note that -1100 is not a good episode return for
+    # Pendulum-v1, we are using it here to shorten the experiment time.
+    run_config=tune.RunConfig(
+        stop={"env_runners/episode_return_mean": -1100.0},
+    ),
+)
+# Run the Tuner and capture the results.
+results = tuner.fit()</t>
+  </si>
+  <si>
+    <t>Ray Tune</t>
   </si>
   <si>
     <r>
@@ -3622,9 +3655,6 @@
 results = tuner.fit()</t>
   </si>
   <si>
-    <t>Ray Tune</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <color rgb="FF1155CC"/>
@@ -3852,6 +3882,1378 @@
   </si>
   <si>
     <t>Command-line reporter</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/facebookresearch/BenchMARL/blob/main/benchmarl/experiment/experiment.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">benchmarl/experiment/experiment.py
+class Experiment(CallbackNotifier):
+    """
+    Main experiment class in BenchMARL.
+An experiment is a training run in which an algorithm, a task, and a model are fixed. </t>
+  </si>
+  <si>
+    <t>train, evaluate, checkpoint</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/facebookresearch/BenchMARL/blob/main/benchmarl/benchmark/benchmark.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">class Benchmark:  
+"""A benchmark.
+Benchmarks are collections of experiments to compare.
+</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/facebookresearch/BenchMARL/blob/main/benchmarl/experiment/experiment.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>class Experiment(CallbackNotifier):
+def run(self):
+        """Run the experiment until completion."""
+        try:
+            seed_everything(self.seed)
+            torch.cuda.empty_cache()
+            self._collection_loop()
+        except KeyboardInterrupt as interrupt:
+            print("\n\nExperiment was closed gracefully\n\n")
+            self.close()
+            raise interrupt
+        except Exception as err:
+            print("\n\nExperiment failed and is closing gracefully\n\n")
+            self.close()
+            raise err</t>
+  </si>
+  <si>
+    <t>execute run() -&gt; get into the train loop, with orchestrator, agent, env</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/facebookresearch/BenchMARL/blob/main/benchmarl/experiment/experiment.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>benchmarl/experiment/experiment.py
+class Experiment(CallbackNotifier):
+def _collection_loop(self):
+ # Training/collection iterations
+# Logging</t>
+  </si>
+  <si>
+    <t>collect data, update policy</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/facebookresearch/BenchMARL/blob/main/benchmarl/run.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> ;
+</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/facebookresearch/BenchMARL/blob/main/benchmarl/hydra_config.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>if _has_hydra:
+    from hydra import compose, initialize, initialize_config_dir
+    from omegaconf import DictConfig, OmegaConf</t>
+  </si>
+  <si>
+    <t>Hydra for flexible and modular configuration</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/facebookresearch/BenchMARL/blob/main/benchmarl/algorithms/iql.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>experiment_config.share_policy_params = True # Policy parameter sharing on
+BenchMARL will automatically group agents based on the VMAS name 
+This allows to stack their data because they are homogeneous.
+Agents from different groups will be kept separate and it is even possible to use different models 
+and algorithms for different groups. 
+It is possible to use different algorithms and models for different agent groups.</t>
+  </si>
+  <si>
+    <t>In algorithms/ folder for each algorithm, for example:
+((all cars togherther, all holonomic together, all differential drive together).
+implementation in algorithm</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/facebookresearch/BenchMARL/blob/main/benchmarl/algorithms/common.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">class Algorithm(ABC):
+    """
+    Abstract class for an algorithm.
+Algorithms. 
+Algorithms are an ensemble of components (e.g., losss, replay buffer) 
+which determine the training strategy. </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/facebookresearch/BenchMARL/tree/main/benchmarl/models</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> ;
+</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/facebookresearch/BenchMARL/blob/main/benchmarl/models/common.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve">  </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Models are neural networks used to process data. 
+They can be used as actors (policies) or, when requested, as critics. 
+We provide a set of base models (layers) and a SequenceModel to concatenate different layers. </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/facebookresearch/BenchMARL/blob/main/benchmarl/environments/common.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>benchmarl/environments/common.py
+torch.data.ReplayBuffer
+A generic, composable replay buffer class.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/facebookresearch/BenchMARL/blob/main/benchmarl/algorithms/common.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>def get_policy_for_loss(self, group: str) -&gt; TensorDictModule:
+        """
+        Get the non-explorative policy for a specific group loss.
+        This function calls the abstract :class:`~benchmarl.algorithms.Algorithm._get_policy_for_loss()` which needs to be implemented.
+        The function will cache the output at the first call and return the cached values in future calls.
+        Args:
+            group (str): agent group of the policy
+        Returns: TensorDictModule representing the policy
+        """
+        if group not in self._policies_for_loss.keys():
+            action_space = self.action_spec[group, "action"]
+            continuous = not isinstance(action_space, (Categorical, OneHot))
+            self._policies_for_loss.update(
+                {
+                    group: self._get_policy_for_loss(
+                        group=group,
+                        continuous=continuous,
+                        model_config=self.model_config,
+                    )
+                }
+            )
+        return self._policies_for_loss[group]</t>
+  </si>
+  <si>
+    <t>inside class Algorithm(ABC), not a seperate module</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/facebookresearch/BenchMARL/blob/main/examples/checkpointing/reload_experiment.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> ;
+</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/facebookresearch/BenchMARL/blob/main/examples/checkpointing/resume_experiment.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>examples/checkpointing/reload_experiment.py
+  # Save the experiment in the current folder
+    experiment_config.save_folder = Path(os.path.dirname(os.path.realpath(__file__)))
+    # Checkpoint at every iteration
+-----
+examples/checkpointing/resume_experiment.py
+reload_experiment_from_file
+ # Now we tell it where to resume from
+    restored_experiment = reload_experiment_from_file(
+        (
+            experiment.folder_name
+            / "checkpoints"
+            / f"checkpoint_{experiment_config.checkpoint_interval}.pt"
+        )
+    )  # Restore from first checkpoint</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/facebookresearch/BenchMARL/blob/main/benchmarl/experiment/logger.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>benchmarl/experiment/logger.py
+class Logger
+ def log_evaluation(
+logger.log_video("eval_video", vid, step=step)
+logger.log_video("eval/video", vid, fps=20, commit=False)</t>
+  </si>
+  <si>
+    <t>inside logger, not a seperate module, only the function</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/facebookresearch/BenchMARL/blob/main/benchmarl/experiment/logger.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>benchmarl/experiment/logger.py
+class Logger
+from torchrl.record import TensorboardLogger
+from torchrl.record.loggers import get_logger
+from torchrl.record.loggers.wandb import WandbLogger</t>
+  </si>
+  <si>
+    <t>BenchMARL is compatible with the TorchRL loggers.</t>
+  </si>
+  <si>
+    <t>TorchRL loggers</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/facebookresearch/BenchMARL/blob/main/benchmarl/eval_results.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/instadeepai/marl-eval/tree/main/marl_eval/plotting_tools</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>benchmarl/eval_results.py
+import collections
+import importlib
+class Plotting:
+Class containing static utilities for plotting in ``marl-eval``.
+from benchmarl.eval_results import load_and_merge_json_dicts, Plotting
+ # Plotting
+    Plotting.performance_profile_figure(
+        environment_comparison_matrix=environment_comparison_matrix
+    )
+    Plotting.aggregate_scores(
+        environment_comparison_matrix=environment_comparison_matrix
+    )
+    Plotting.environemnt_sample_efficiency_curves(
+        sample_effeciency_matrix=sample_efficiency_matrix
+    )
+    Plotting.task_sample_efficiency_curves(
+        processed_data=processed_data, env="vmas", task="navigation"
+    )
+    Plotting.probability_of_improvement(
+        environment_comparison_matrix,
+        algorithms_to_compare=[["qmix", "mappo"]],
+    )
+    plt.show()
+-----
+marl_eval/plotting_tools
+from marl_eval.plotting_tools.plotting import (
+        aggregate_scores,
+        performance_profiles,
+        plot_single_task,
+        probability_of_improvement,
+        sample_efficiency_curves,
+    )
+    from marl_eval.utils.data_processing_utils import (
+        create_matrices_for_rliable,
+        data_process_pipeline,
+    )
+    from matplotlib import pyplot as plt</t>
+  </si>
+  <si>
+    <t>Plotting</t>
+  </si>
+  <si>
+    <t>marl_eval/plotting_tools</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/instadeepai/Mava/tree/develop/mava/systems</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/instadeepai/Mava/blob/develop/mava/systems/ppo/anakin/ff_ippo.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>def run_experiment(_config: DictConfig) -&gt; float:
+    """Runs experiment."""
+setup environment, logging, checkpoint, 
+learn, actor_network, learner_state = learner_setup(
+        env, (key, actor_net_key, critic_net_key), config
+    )
+learn, evaluate, output</t>
+  </si>
+  <si>
+    <t>mava/systems
+(each algorithm one file)
+For example the link here.
+mix responsibilities with the Framework Orchestrator.
+The Experiment Manager sets up the Utilities components
+(e.g., Checkpoint Manager)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/instadeepai/Mava/tree/develop/mava/systems</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/instadeepai/Mava/blob/develop/mava/systems/ppo/anakin/ff_ippo.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>mava/systems
+(each algorithm one file)
+For example the link here.
+learn, evaluate, output
+mix responsibilities with the Experiment Manager.
+the Framework Orchestrator sets up the framework components (e.g., Agent and Lifecycle Manager), and orchestrates their operation.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/instadeepai/Mava/blob/develop/mava/systems/gpo/anakin/rec_magpo.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>def _env_step(
+            learner_state: LearnerState, _: Any
+        ) -&gt; Tuple[LearnerState, Tuple[Transition, Metrics]]:
+            """Step the environment."""</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> inside Algorithm, for example the link here,
+step through, info change between env and agent</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/instadeepai/Mava/tree/develop</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> ;
+</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/instadeepai/Mava/blob/develop/mava/systems/ppo/anakin/ff_ippo.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Mava makes use of Hydra for config management. In order to see our default system configs please see the mava/configs/ directory. A benefit of Hydra is that configs can either be set in config yaml files or overwritten from the terminal on the fly. 
+----
+from omegaconf import DictConfig, OmegaConf
+import hydra
+Hydra's configuration object is an instance of OmegaConf's DictConfig.
+config: DictConfig = OmegaConf.create(config)
+def hydra_entry_point(cfg: DictConfig) -&gt; float:
+    """Experiment entry point."""
+    # Allow dynamic attributes.
+    OmegaConf.set_struct(cfg, False)
+    # Run experiment.
+    eval_performance = run_experiment(cfg)
+    print(f"{Fore.CYAN}{Style.BRIGHT}IPPO experiment completed{Style.RESET_ALL}")
+    return eval_performance
+if __name__ == "__main__":
+    hydra_entry_point()
+</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/instadeepai/Mava/blob/develop/mava/systems/sac/anakin/ff_isac.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t># Number of env steps before evaluating/logging.
+    steps_per_rollout = int(cfg.system.total_timesteps // cfg.arch.num_evaluation)
+    # Multiplier for a single env/learn step in an anakin system
+    anakin_steps = cfg.arch.n_devices * cfg.system.update_batch_size
+    # Number of env steps in one anakin style update.
+    anakin_act_steps = anakin_steps * cfg.arch.num_envs * cfg.system.rollout_length
+    # Number of steps to do in the scanned update method (how many anakin steps).
+    cfg.system.scan_steps = int(steps_per_rollout / anakin_act_steps)
+# Distribute params and opt states across all devices
+    params = replicate(params)
+    opt_states = replicate(opt_states)</t>
+  </si>
+  <si>
+    <t>support distribution, but not a complete module.
+Anakin architecture (Hessel et al., 2021) for scalable distributed system training on hardware
+accelerators
+Mava supports both Podracer architectures for scaling RL systems. The first of these is Anakin, which can be used when environments are written in JAX. This enables end-to-end JIT compilation of the full MARL training loop for fast experiment run times on hardware accelerators. The second is Sebulba, which can be used when environments are not written in JAX. Sebulba is particularly useful when running RL experiments where a hardware accelerator can interact with many CPU cores at a time.</t>
+  </si>
+  <si>
+    <t>https://github.com/instadeepai/Mava/blob/develop/mava/systems/ppo/anakin/rec_mappo.py</t>
+  </si>
+  <si>
+    <t># Step environment for rollout length
+        learner_state, (traj_batch, episode_metrics) = jax.lax.scan(
+            _env_step, learner_state, length=config.system.rollout_length
+        )
+        # Calculate advantage
+        params, opt_states, key, env_state, last_timestep, last_done, updated_hstates = (
+            learner_state
+        )</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/instadeepai/Mava/tree/develop/mava/networks</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/instadeepai/Mava/blob/develop/mava/networks/base.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>Actor(nn.Module)/Critic()
+from mava.networks.base import (
+    FeedForwardActor,
+    FeedForwardQNet,
+    FeedForwardValueNet,
+    RecQNetwork,
+    RecurrentActor,
+    RecurrentValueNet,
+    ScannedRNN,
+)</t>
+  </si>
+  <si>
+    <t>only the complete network module, seperate implementations, implement nn,Module, but all the function approcximator logics are merged into the each single algorithm implementaion. not modular.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/instadeepai/Mava/blob/develop/mava/systems/sac/anakin/ff_isac.p </t>
+  </si>
+  <si>
+    <t>import flashbax as fbx
+from colorama import Fore, Style
+from flashbax.buffers.flat_buffer import TrajectoryBuffer
+ # Create replay buffer
+    init_transition = Transition(
+        obs=obs,
+        action=acts,
+        reward=jnp.zeros((n_agents,), dtype=float),
+        done=jnp.zeros((n_agents,), dtype=bool),
+        next_obs=obs,
+    )
+    rb = fbx.make_item_buffer(
+        max_length=int(cfg.system.buffer_size),
+        min_length=int(cfg.system.explore_steps),
+        sample_batch_size=int(cfg.system.batch_size),
+        add_batches=True,
+    )
+    buffer_state = replicate(rb.init(init_transition))</t>
+  </si>
+  <si>
+    <t>FlashBax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/instadeepai/Mava/blob/develop/mava/systems/sac/anakin/ff_isac.py  </t>
+  </si>
+  <si>
+    <t>data = rb.sample(buffer_state, buff_key).experience
+params, opt_states, q_loss_info = update_q(params, opt_states, data, q_key)
+# Sample and learn
+        learn_state = (buffer_state, params, opt_states, t, learn_key)
+        (buffer_state, params, opt_states, _, _), losses = scanned_train(learn_state)
+        t += cfg.arch.num_envs * cfg.system.rollout_length
+        return (
+            LearnerState(next_obs, env_state, buffer_state, params, opt_states, t, key),
+            (metrics, losses),
+        )
+learner_setup
+def get_learner_fn(
+    env: jumanji.Environment,
+    apply_fns: Tuple[ActorApply, CriticApply],
+    update_fns: Tuple[optax.TransformUpdateFn, optax.TransformUpdateFn],
+    config: DictConfig,
+) -&gt; LearnerFn[LearnerState]:
+    """Get the learner function."""
+    # Unpack apply and update functions.
+    actor_apply_fn, critic_apply_fn = apply_fns
+    actor_update_fn, critic_update_fn = update_fns
+    def _update_step(learner_state: LearnerState, _: Any) -&gt; Tuple[LearnerState, Tuple]:
+        """A single update of the network.
+ def learner_fn(learner_state: LearnerState) -&gt; ExperimentOutput[LearnerState]:
+        """Learner function.</t>
+  </si>
+  <si>
+    <t>all the learner logics are merged into the each single algorithm implementaion. 
+not modular.
+(learner_func here, but no learner)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/instadeepai/Mava/blob/develop/mava/utils/checkpointing.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>mava/utils/checkpointing.py
+class Checkpointer:
+Model checkpointer for saving and restoring the `learner_state`.
+import orbax.checkpoint</t>
+  </si>
+  <si>
+    <t>Orbax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/instadeepai/Mava/blob/develop/mava/utils/logger.py </t>
+  </si>
+  <si>
+    <t>mava/utils/logger.py
+class MavaLogger:
+    def __init__(
+        self,
+        config: DictConfig,
+        custom_metrics_fn: Callable[[Metrics], Metrics] = winrate_custom_metric,
+    ) -&gt; None:
+        """The main logger for Mava systems.
+class NeptuneLogger(BaseLogger):
+    def __init__(
+        self,
+        base_exp_path: PathLike,
+        unique_token: str,
+        system_name: str,
+        project: str,
+        tag: list[str],
+        group_tag: list[str],
+        detailed_logging: bool,
+        architecture_name: str,
+        upload_json_data: bool,
+        run_id: str | None = None,
+    ) -&gt; None:
+        """
+        Initialize neptune.ai logger for experiment tracking.
+class TensorboardLogger(BaseLogger):
+    def __init__(self, base_exp_path: PathLike, unique_token: str, system_name: str) -&gt; None:
+        """
+        Initialize TensorBoard logger for visualization.
+        Args:
+            base_exp_path: Base path where logs will be stored
+            unique_token: Unique identifier string for this run
+            system_name: Name of the system/algorithm being logged
+        """</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neptune, Tensorboard
+</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/instadeepai/Mava/blob/develop/mava/utils/logger.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>class TensorboardLogger(BaseLogger):
+    def __init__(self, base_exp_path: PathLike, unique_token: str, system_name: str) -&gt; None:
+        """
+        Initialize TensorBoard logger for visualization.</t>
+  </si>
+  <si>
+    <t>tensorboard for visualization</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/google/dopamine/blob/master/dopamine/discrete_domains/run_experiment.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>dopamine/discrete_domains/run_experiment.py
+@gin.configurable
+class Runner(object):
+  """Object that handles running Dopamine experiments.
+Here we use the term 'experiment' to mean simulating interactions between the agent and the environment and reporting some statistics pertaining to these interactions.</t>
+  </si>
+  <si>
+    <t>create checkpoint, logging
+save, summarize
+mix responsibilities with the Framework Orchestrator.
+The Experiment Manager sets up the Utilities components
+(e.g., Checkpoint Manager)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/google/dopamine/blob/master/dopamine/discrete_domains/run_experiment.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>create env, agent,
+initialize, run
+mix responsibilities with the Experiment Manager.
+the Framework Orchestrator sets up the framework components (e.g., Agent and Lifecycle Manager), and orchestrates their operation.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/google/dopamine/blob/master/dopamine/discrete_domains/run_experiment.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/google/dopamine/blob/master/dopamine/jax/agents/full_rainbow/full_rainbow_agent.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>run
+def _run_train_phase(self, statistics):
+    """Run training phase.
+def _run_eval_phase(self, statistics):
+    """Run evaluation phase.
+-----
+def _train_step(self):
+    """Runs a single training step.
+    Runs training if both:
+      (1) A minimum number of frames have been added to the replay buffer.
+      (2) `training_steps` is a multiple of `update_period`.</t>
+  </si>
+  <si>
+    <t>run call agent.train_step
+train_step: agent &lt;-&gt; env</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/google/dopamine/blob/master/dopamine/discrete_domains/run_experiment.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>def load_gin_configs(gin_files, gin_bindings):
+  """Loads gin configuration files.
+  Args:
+    gin_files: list, of paths to the gin configuration files for this
+      experiment.
+    gin_bindings: list, of gin parameter bindings to override the values in the
+      config files.
+  """
+  gin.parse_config_files_and_bindings(
+      gin_files, bindings=gin_bindings, skip_unknown=False
+  )
+Gin Config, lightweight configuration framework
+The whole of Dopamine is easily configured using the gin configuration framework.</t>
+  </si>
+  <si>
+    <t>Gin</t>
+  </si>
+  <si>
+    <t>https://github.com/google/dopamine/tree/master/dopamine/jax/agents</t>
+  </si>
+  <si>
+    <t>class JaxDQNAgent(object):
+  """A JAX implementation of the DQN agent."""</t>
+  </si>
+  <si>
+    <t>for each diffeernt type algorithm they have different agent
+The agent class, in dopamine/agents.
+for example, DQNAgent</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/google/dopamine/blob/master/dopamine/jax/agents/dqn/dqn_agent.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>agent.def _record_observation(self, observation):
+    """Records an observation and update state.
+def select_action(
+def step(self, reward, observation):
+    """Returns the agent's next action and update agent's state.</t>
+  </si>
+  <si>
+    <t>functions have the responsibilities of Function Approximator, but not a seperate module, they are merged into Agent.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/google/dopamine/blob/master/dopamine/jax/replay_memory/replay_buffer.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>dopamine/jax/replay_memory/replay_buffer.py
+class ReplayBuffer(checkpointers.Checkpointable, Generic[ReplayElementT]):
+  """A Jax re-implementation of the Dopamine Replay Buffer.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/google/dopamine/blob/master/dopamine/labs/offline_rl/jax/offline_dqn_agent.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>def step(self, reward, observation):
+    """Returns the agent's next action and update agent's state.</t>
+  </si>
+  <si>
+    <t>functions have the responsibilities of Learner, but not a seperate module, they are merged into Agent.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/google/dopamine/blob/master/dopamine/discrete_domains/checkpointer.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>dopamine/discrete_domains/checkpointer.py
+"""A checkpointing mechanism for Dopamine agents.
+from absl import logging
+from dopamine.discrete_domains import atari_lib
+from dopamine.discrete_domains import checkpointer
+from dopamine.discrete_domains import iteration_statistics
+from dopamine.discrete_domains import logger
+class Checkpointer(object):
+  """Class for managing checkpoints for Dopamine agents."""</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/google/dopamine/blob/master/dopamine/utils/agent_visualizer.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>class AgentVisualizer(object):
+  """Code to visualize an agent's behaviour."""
+  def __init__(
+      self,
+      record_path,
+      plotters,
+      screen_width=160,
+      screen_height=210,
+      render_rate=1,
+      file_types=('png', ''),
+      filename_format='frame_{:06d}',
+  ):
+    """Constructor for the AgentVisualizer class.
+This class generates a series of images built by a set of Plotters. These images are then saved to disk.
+It can optionally generate a video by concatenating all the images with ffmpeg.</t>
+  </si>
+  <si>
+    <t>This class generates a series of images built by a set of Plotters. These images are then saved to disk.
+It can optionally generate a video by concatenating all the images with ffmpeg.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/google/dopamine/blob/master/dopamine/discrete_domains/logger.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>dopamine/discrete_domains/logger.py
+class Logger(object):
+  """Class for maintaining a dictionary of data to log."""</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/google/dopamine/blob/master/dopamine/continuous_domains/run_experiment.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>def _save_tensorboard_summaries(
+      self, iteration, num_episodes, average_reward, average_steps_per_second
+  ):
+    """Save statistics as tensorboard summaries."""
+    if self._summary_writer is None:
+      return
+    if self._sess is None:
+      with self._summary_writer.as_default():
+        tf.summary.scalar('Train/NumEpisodes', num_episodes, step=iteration)
+        tf.summary.scalar(
+            'Train/AverageReturns', average_reward, step=iteration
+        )
+        tf.summary.scalar(
+            'Train/AverageStepsPerSecond',
+            average_steps_per_second,
+            step=iteration,
+        )
+      self._summary_writer.flush()
+    else:
+      summary = tf.compat.v1.Summary(
+          value=[
+              tf.compat.v1.Summary.Value(
+                  tag='Train/NumEpisodes', simple_value=num_episodes
+              ),
+              tf.compat.v1.Summary.Value(
+                  tag='Train/AverageReturns', simple_value=average_reward
+              ),
+              tf.compat.v1.Summary.Value(
+                  tag='Train/AverageStepsPerSecond',
+                  simple_value=average_steps_per_second,
+              ),
+          ]
+      )
+      self._summary_writer.add_summary(summary, iteration)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/thu-ml/tianshou/blob/master/tianshou/highlevel/experiment.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>tianshou/highlevel/experiment.py
+The experiment module provides high-level interfaces 
+for setting up and running reinforcement learning experiments.</t>
+  </si>
+  <si>
+    <t>setup, checkpoint, run, collect result,
+persistence and the overall experiment flow</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/thu-ml/tianshou/blob/master/tianshou/trainer.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">tianshou/trainer.py
+This module contains Tianshou's trainer classes, which orchestrate the training and call upon an RL algorithm's
+specific network updating logic to perform the actual gradient updates.
+The base class already implements the fundamental epoch logic and fully implements the test step
+logic, which is common to all trainers. </t>
+  </si>
+  <si>
+    <t>controls fundamental training parameters, such as the total number of epochs we run the experiment for</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/thu-ml/tianshou/blob/master/tianshou/trainer.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>tianshou/trainer.py
+def run(
+        self, reset_collectors: bool = True, reset_collector_buffers: bool = False
+    ) -&gt; InfoStats:
+        """Runs the training process with the configuration given at construction.
+def _training_step(self) -&gt; _TrainingStepResult:
+        """Performs one training step."""</t>
+  </si>
+  <si>
+    <t>run: world.trainer.run() 
+(env &lt;-&gt; agent, function indie the framework orchestrator, not a seperate module here)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/thu-ml/tianshou/blob/master/tianshou/highlevel/config.py </t>
+  </si>
+  <si>
+    <t>tianshou/config.py
+tianshou/highlevel/config.py
+class TrainingConfig(ToStringMixin):
+    """Training configuration."""</t>
+  </si>
+  <si>
+    <t>https://github.com/thu-ml/tianshou/blob/master/tianshou/algorithm/multiagent/marl.py</t>
+  </si>
+  <si>
+    <t>tianshou/algorithm/multiagent/marl.py
+class MultiAgentPolicy(Policy):
+def forward(  # type: ignore
+        self,
+        batch: Batch,
+        state: dict | Batch | None = None,
+        **kwargs: Any,
+    ) -&gt; Batch:
+        """Dispatch batch data from obs.agent_id to every policy's forward.
+preprocess batch, update batch
+ for agent_id, policy in self.policies.items():
+            # This part of code is difficult to understand.
+            # Let's follow an example with two agents
+            # batch.obs.agent_id is [1, 2, 1, 2, 1, 2] (with batch_size == 6)
+            # each agent plays for three transitions
+            # agent_index for agent 1 is [0, 2, 4]
+            # agent_index for agent 2 is [1, 3, 5]
+            # we separate the transition of each agent according to agent_id
+            agent_index = np.nonzero(batch.obs.agent_id == agent_id)[0]</t>
+  </si>
+  <si>
+    <t>Dispatch batch data from obs.agent_id to every policy's forward.
+separate the transition of each agent according to agent_id
+policy coordination for MARL</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/thu-ml/tianshou/tree/master/tianshou/algorithm  ;
+https://github.com/thu-ml/tianshou/blob/master/tianshou/algorithm/algorithm_base.py</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF000000"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>class Algorithm(torch.nn.Module, Generic[TPolicy, TTrainerParams], ABC):</t>
+  </si>
+  <si>
+    <t>tianshou/algorithm (different algorithms in the folder)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/thu-ml/tianshou/blob/master/tianshou/algorithm/algorithm_base.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>class Policy(nn.Module, ABC):
+    """Represents a policy, which provides the fundamental mapping from observations to actions."""</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/thu-ml/tianshou/blob/master/tianshou/data/buffer</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> ;
+</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/thu-ml/tianshou/blob/master/tianshou/data/buffer/buffer_base.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>class ReplayBuffer:
+    """:class:`~tianshou.data.ReplayBuffer` stores data generated from interaction between the policy and environment.
+    ReplayBuffer can be considered as a specialized form (or management) of Batch. It
+    stores all the data in a batch with circular-queue style.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/thu-ml/tianshou/blob/master/tianshou/algorithm/algorithm_base.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>class Optimizer:
+        """Wrapper for a torch optimizer that optionally performs gradient clipping."""</t>
+  </si>
+  <si>
+    <t>Optimizer has the same role as Learner</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/thu-ml/tianshou/blob/master/tianshou/highlevel/persistence.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>tianshou/highlevel/persistence.py
+def get_save_checkpoint_fn(self, world: World) -&gt; Callable[[int, int, int], str] | None:
+        if not self.enabled:
+            return None
+        def save_checkpoint_fn(epoch: int, env_step: int, gradient_step: int) -&gt; str:</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://github.com/thu-ml/tianshou/blob/master/tianshou/highlevel/logger.py</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>tianshou/highlevel/logger.py
+from tianshou.utils import BaseLogger, TensorboardLogger, WandbLogger
+"""A logger that relies on tensorboard SummaryWriter by default to visualize and log statistics.</t>
+  </si>
+  <si>
+    <t>TensorboardLogger
+WandbLogger</t>
+  </si>
+  <si>
+    <t>TensorboardLogger</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/thu-ml/tianshou/blob/master/tianshou/highlevel/logger.py </t>
+  </si>
+  <si>
+    <t>tensorboard SummaryWriter</t>
+  </si>
+  <si>
+    <t>Tensorboard SummaryWriter</t>
   </si>
 </sst>
 </file>
@@ -33343,7 +34745,7 @@
     <col customWidth="1" min="3" max="3" width="19.13"/>
     <col customWidth="1" min="4" max="4" width="15.88"/>
     <col customWidth="1" min="5" max="5" width="26.25"/>
-    <col customWidth="1" min="6" max="6" width="35.38"/>
+    <col customWidth="1" min="6" max="6" width="47.63"/>
     <col customWidth="1" min="7" max="7" width="36.38"/>
     <col customWidth="1" min="8" max="8" width="18.13"/>
   </cols>
@@ -37280,7 +38682,9 @@
       <c r="G93" s="11" t="s">
         <v>201</v>
       </c>
-      <c r="H93" s="9"/>
+      <c r="H93" s="11" t="s">
+        <v>202</v>
+      </c>
       <c r="I93" s="9"/>
       <c r="J93" s="9"/>
       <c r="K93" s="9"/>
@@ -37558,14 +38962,14 @@
         <v>external</v>
       </c>
       <c r="E100" s="10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F100" s="11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="G100" s="9"/>
       <c r="H100" s="11" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="I100" s="9"/>
       <c r="J100" s="9"/>
@@ -37604,13 +39008,13 @@
         <v>implicit</v>
       </c>
       <c r="E101" s="10" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F101" s="11" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G101" s="11" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="H101" s="9"/>
       <c r="I101" s="9"/>
@@ -37851,10 +39255,10 @@
         <v>explicit</v>
       </c>
       <c r="E107" s="10" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F107" s="11" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G107" s="9"/>
       <c r="H107" s="9"/>
@@ -37895,10 +39299,10 @@
         <v>explicit</v>
       </c>
       <c r="E108" s="10" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F108" s="11" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="G108" s="9"/>
       <c r="H108" s="9"/>
@@ -37939,16 +39343,16 @@
         <v>external</v>
       </c>
       <c r="E109" s="10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F109" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G109" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="H109" s="11" t="s">
         <v>214</v>
-      </c>
-      <c r="H109" s="11" t="s">
-        <v>213</v>
       </c>
       <c r="I109" s="9"/>
       <c r="J109" s="9"/>
@@ -37987,13 +39391,13 @@
         <v>explicit</v>
       </c>
       <c r="E110" s="10" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F110" s="11" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G110" s="11" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H110" s="9"/>
       <c r="I110" s="9"/>
@@ -38074,13 +39478,13 @@
         <v>implicit</v>
       </c>
       <c r="E112" s="10" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F112" s="11" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="G112" s="11" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="H112" s="9"/>
       <c r="I112" s="9"/>
@@ -38120,10 +39524,10 @@
         <v>explicit</v>
       </c>
       <c r="E113" s="10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F113" s="11" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="G113" s="9"/>
       <c r="H113" s="9"/>
@@ -38164,10 +39568,10 @@
         <v>explicit</v>
       </c>
       <c r="E114" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F114" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G114" s="9"/>
       <c r="H114" s="9"/>
@@ -38208,10 +39612,10 @@
         <v>explicit</v>
       </c>
       <c r="E115" s="10" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F115" s="11" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="G115" s="9"/>
       <c r="H115" s="9"/>
@@ -38813,13 +40217,13 @@
         <v>explicit</v>
       </c>
       <c r="E130" s="10" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F130" s="11" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G130" s="11" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H130" s="9"/>
       <c r="I130" s="9"/>
@@ -38859,13 +40263,13 @@
         <v>explicit</v>
       </c>
       <c r="E131" s="10" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F131" s="11" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="G131" s="11" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="H131" s="9"/>
       <c r="I131" s="9"/>
@@ -38905,16 +40309,16 @@
         <v>external</v>
       </c>
       <c r="E132" s="10" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F132" s="11" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G132" s="11" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H132" s="11" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I132" s="9"/>
       <c r="J132" s="9"/>
@@ -38953,13 +40357,13 @@
         <v>implicit</v>
       </c>
       <c r="E133" s="10" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F133" s="11" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="G133" s="11" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="H133" s="9"/>
       <c r="I133" s="9"/>
@@ -39080,13 +40484,13 @@
         <v>explicit</v>
       </c>
       <c r="E136" s="15" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F136" s="11" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="G136" s="11" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="H136" s="9"/>
       <c r="I136" s="9"/>
@@ -39166,10 +40570,10 @@
         <v>explicit</v>
       </c>
       <c r="E138" s="10" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F138" s="11" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="G138" s="9"/>
       <c r="H138" s="9"/>
@@ -39771,10 +41175,10 @@
         <v>explicit</v>
       </c>
       <c r="E153" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F153" s="11" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G153" s="9"/>
       <c r="H153" s="9"/>
@@ -39815,13 +41219,13 @@
         <v>explicit</v>
       </c>
       <c r="E154" s="10" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F154" s="11" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G154" s="11" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="H154" s="9"/>
       <c r="I154" s="9"/>
@@ -39861,16 +41265,16 @@
         <v>external</v>
       </c>
       <c r="E155" s="10" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F155" s="11" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="G155" s="11" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="H155" s="11" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="I155" s="9"/>
       <c r="J155" s="9"/>
@@ -39909,13 +41313,13 @@
         <v>explicit</v>
       </c>
       <c r="E156" s="10" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F156" s="11" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="G156" s="11" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="H156" s="9"/>
       <c r="I156" s="9"/>
@@ -40036,10 +41440,10 @@
         <v>explicit</v>
       </c>
       <c r="E159" s="10" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F159" s="11" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="G159" s="9"/>
       <c r="H159" s="9"/>
@@ -40080,10 +41484,10 @@
         <v>explicit</v>
       </c>
       <c r="E160" s="10" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F160" s="11" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="G160" s="9"/>
       <c r="H160" s="9"/>
@@ -40124,10 +41528,10 @@
         <v>explicit</v>
       </c>
       <c r="E161" s="10" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F161" s="11" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="G161" s="9"/>
       <c r="H161" s="9"/>
@@ -40729,10 +42133,10 @@
         <v>explicit</v>
       </c>
       <c r="E176" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F176" s="5" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="G176" s="1"/>
       <c r="H176" s="9"/>
@@ -40773,13 +42177,13 @@
         <v>explicit</v>
       </c>
       <c r="E177" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="F177" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="F177" s="5" t="s">
-        <v>264</v>
-      </c>
       <c r="G177" s="5" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H177" s="9"/>
       <c r="I177" s="9"/>
@@ -40819,16 +42223,16 @@
         <v>external</v>
       </c>
       <c r="E178" s="14" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F178" s="5" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="G178" s="5" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="H178" s="11" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="I178" s="9"/>
       <c r="J178" s="9"/>
@@ -40867,13 +42271,13 @@
         <v>implicit</v>
       </c>
       <c r="E179" s="16" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F179" s="5" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G179" s="5" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="H179" s="9"/>
       <c r="I179" s="9"/>
@@ -40954,13 +42358,13 @@
         <v>implicit</v>
       </c>
       <c r="E181" s="10" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F181" s="11" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G181" s="11" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="H181" s="9"/>
       <c r="I181" s="9"/>
@@ -41000,10 +42404,10 @@
         <v>explicit</v>
       </c>
       <c r="E182" s="10" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="F182" s="11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="G182" s="9"/>
       <c r="H182" s="9"/>
@@ -41044,10 +42448,10 @@
         <v>explicit</v>
       </c>
       <c r="E183" s="10" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F183" s="11" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G183" s="9"/>
       <c r="H183" s="9"/>
@@ -41088,10 +42492,10 @@
         <v>explicit</v>
       </c>
       <c r="E184" s="15" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F184" s="11" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G184" s="9"/>
       <c r="H184" s="9"/>
@@ -41693,10 +43097,10 @@
         <v>explicit</v>
       </c>
       <c r="E199" s="15" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F199" s="11" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G199" s="9"/>
       <c r="H199" s="9"/>
@@ -41737,13 +43141,13 @@
         <v>explicit</v>
       </c>
       <c r="E200" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="F200" s="11" t="s">
         <v>284</v>
       </c>
-      <c r="F200" s="11" t="s">
-        <v>283</v>
-      </c>
       <c r="G200" s="11" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="H200" s="9"/>
       <c r="I200" s="9"/>
@@ -41783,13 +43187,13 @@
         <v>implicit</v>
       </c>
       <c r="E201" s="10" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F201" s="11" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G201" s="11" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="H201" s="9"/>
       <c r="I201" s="9"/>
@@ -41869,10 +43273,10 @@
         <v>implicit</v>
       </c>
       <c r="E203" s="10" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="F203" s="11" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="G203" s="9"/>
       <c r="H203" s="9"/>
@@ -41954,10 +43358,10 @@
         <v>explicit</v>
       </c>
       <c r="E205" s="10" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F205" s="11" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="G205" s="9"/>
       <c r="H205" s="9"/>
@@ -42038,10 +43442,10 @@
         <v>explicit</v>
       </c>
       <c r="E207" s="10" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F207" s="11" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="G207" s="9"/>
       <c r="H207" s="9"/>
@@ -42162,13 +43566,13 @@
         <v>implicit</v>
       </c>
       <c r="E210" s="10" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F210" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G210" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="H210" s="9"/>
       <c r="I210" s="9"/>
@@ -42288,13 +43692,13 @@
         <v>implicit</v>
       </c>
       <c r="E213" s="10" t="s">
+        <v>299</v>
+      </c>
+      <c r="F213" s="11" t="s">
+        <v>297</v>
+      </c>
+      <c r="G213" s="11" t="s">
         <v>298</v>
-      </c>
-      <c r="F213" s="11" t="s">
-        <v>296</v>
-      </c>
-      <c r="G213" s="11" t="s">
-        <v>297</v>
       </c>
       <c r="H213" s="9"/>
       <c r="I213" s="9"/>
@@ -42334,13 +43738,13 @@
         <v>implicit</v>
       </c>
       <c r="E214" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F214" s="11" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="G214" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="H214" s="9"/>
       <c r="I214" s="9"/>
@@ -42501,13 +43905,13 @@
         <v>explicit</v>
       </c>
       <c r="E218" s="15" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F218" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="G218" s="11" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="H218" s="9"/>
       <c r="I218" s="9"/>
@@ -42547,10 +43951,10 @@
         <v>explicit</v>
       </c>
       <c r="E219" s="10" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="F219" s="11" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="G219" s="9"/>
       <c r="H219" s="9"/>
@@ -42591,13 +43995,13 @@
         <v>explicit</v>
       </c>
       <c r="E220" s="10" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="F220" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="G220" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H220" s="9"/>
       <c r="I220" s="9"/>
@@ -42637,13 +44041,13 @@
         <v>implicit</v>
       </c>
       <c r="E221" s="15" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="F221" s="11" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="G221" s="11" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="H221" s="9"/>
       <c r="I221" s="9"/>
@@ -42843,10 +44247,10 @@
         <v>explicit</v>
       </c>
       <c r="E226" s="10" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="F226" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="G226" s="9"/>
       <c r="H226" s="9"/>
@@ -42968,10 +44372,10 @@
         <v>explicit</v>
       </c>
       <c r="E229" s="10" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F229" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="G229" s="9"/>
       <c r="H229" s="9"/>
@@ -43012,10 +44416,10 @@
         <v>explicit</v>
       </c>
       <c r="E230" s="10" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F230" s="11" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="G230" s="9"/>
       <c r="H230" s="9"/>
@@ -43056,14 +44460,14 @@
         <v>external</v>
       </c>
       <c r="E231" s="10" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="F231" s="11" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G231" s="11"/>
       <c r="H231" s="11" t="s">
-        <v>321</v>
+        <v>202</v>
       </c>
       <c r="I231" s="9"/>
       <c r="J231" s="9"/>
@@ -44179,10 +45583,16 @@
         <f t="array" ref="D257">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A256)-1, 23)+1, INT((ROW(A256)-1)/23)+1)</f>
         <v>external</v>
       </c>
-      <c r="E257" s="9"/>
-      <c r="F257" s="9"/>
+      <c r="E257" s="10" t="s">
+        <v>345</v>
+      </c>
+      <c r="F257" s="11" t="s">
+        <v>346</v>
+      </c>
       <c r="G257" s="9"/>
-      <c r="H257" s="9"/>
+      <c r="H257" s="11" t="s">
+        <v>347</v>
+      </c>
       <c r="I257" s="9"/>
       <c r="J257" s="9"/>
       <c r="K257" s="9"/>
@@ -44260,13 +45670,13 @@
         <v>implicit</v>
       </c>
       <c r="E259" s="10" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="F259" s="11" t="s">
         <v>343</v>
       </c>
       <c r="G259" s="11" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="H259" s="9"/>
       <c r="I259" s="9"/>
@@ -44306,13 +45716,13 @@
         <v>explicit</v>
       </c>
       <c r="E260" s="10" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="F260" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="G260" s="11" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="H260" s="9"/>
       <c r="I260" s="9"/>
@@ -44352,10 +45762,10 @@
         <v>explicit</v>
       </c>
       <c r="E261" s="10" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="F261" s="11" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="G261" s="9"/>
       <c r="H261" s="9"/>
@@ -44396,13 +45806,13 @@
         <v>implicit</v>
       </c>
       <c r="E262" s="10" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="F262" s="11" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="G262" s="11" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="H262" s="9"/>
       <c r="I262" s="9"/>
@@ -44443,14 +45853,14 @@
         <v>external</v>
       </c>
       <c r="E263" s="10" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="F263" s="11" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="G263" s="9"/>
       <c r="H263" s="11" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="I263" s="9"/>
       <c r="J263" s="9"/>
@@ -44489,10 +45899,10 @@
         <v>explicit</v>
       </c>
       <c r="E264" s="10" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="F264" s="11" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="G264" s="9"/>
       <c r="H264" s="9"/>
@@ -44533,13 +45943,13 @@
         <v>explicit</v>
       </c>
       <c r="E265" s="10" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="F265" s="11" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="G265" s="11" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="H265" s="9"/>
       <c r="I265" s="9"/>
@@ -44579,10 +45989,10 @@
         <v>explicit</v>
       </c>
       <c r="E266" s="15" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="F266" s="11" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="G266" s="9"/>
       <c r="H266" s="9"/>
@@ -44623,13 +46033,13 @@
         <v>explicit</v>
       </c>
       <c r="E267" s="10" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="F267" s="11" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="G267" s="11" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="H267" s="9"/>
       <c r="I267" s="9"/>
@@ -44829,10 +46239,10 @@
         <v>explicit</v>
       </c>
       <c r="E272" s="10" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="F272" s="11" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="G272" s="9"/>
       <c r="H272" s="9"/>
@@ -44874,10 +46284,10 @@
         <v>not implemented</v>
       </c>
       <c r="E273" s="10" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="F273" s="11" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="G273" s="9"/>
       <c r="H273" s="9"/>
@@ -45038,10 +46448,10 @@
         <v>explicit</v>
       </c>
       <c r="E277" s="10" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="F277" s="11" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="G277" s="9"/>
       <c r="H277" s="9"/>
@@ -45122,13 +46532,13 @@
         <v>implicit</v>
       </c>
       <c r="E279" s="10" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="F279" s="11" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="G279" s="11" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="H279" s="9"/>
       <c r="I279" s="9"/>
@@ -45248,13 +46658,13 @@
         <v>implicit</v>
       </c>
       <c r="E282" s="10" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="F282" s="11" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="G282" s="11" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="H282" s="9"/>
       <c r="I282" s="9"/>
@@ -45294,10 +46704,10 @@
         <v>explicit</v>
       </c>
       <c r="E283" s="10" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="F283" s="11" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="G283" s="9"/>
       <c r="H283" s="9"/>
@@ -45419,16 +46829,16 @@
         <v>external</v>
       </c>
       <c r="E286" s="10" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="F286" s="11" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="G286" s="11" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="H286" s="11" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="I286" s="9"/>
       <c r="J286" s="9"/>
@@ -45467,10 +46877,10 @@
         <v>explicit</v>
       </c>
       <c r="E287" s="10" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="F287" s="11" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="G287" s="9"/>
       <c r="H287" s="9"/>
@@ -45511,13 +46921,13 @@
         <v>explicit</v>
       </c>
       <c r="E288" s="17" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="F288" s="11" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="G288" s="11" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="H288" s="9"/>
       <c r="I288" s="9"/>
@@ -45557,16 +46967,16 @@
         <v>external</v>
       </c>
       <c r="E289" s="10" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="F289" s="11" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="G289" s="11" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="H289" s="11" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="I289" s="9"/>
       <c r="J289" s="9"/>
@@ -45605,10 +47015,10 @@
         <v>explicit</v>
       </c>
       <c r="E290" s="15" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="F290" s="11" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="G290" s="9"/>
       <c r="H290" s="9"/>
@@ -45809,10 +47219,10 @@
         <v>explicit</v>
       </c>
       <c r="E295" s="10" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="F295" s="11" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="G295" s="9"/>
       <c r="H295" s="9"/>
@@ -45934,10 +47344,10 @@
         <v>explicit</v>
       </c>
       <c r="E298" s="10" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="F298" s="11" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="G298" s="9"/>
       <c r="H298" s="9"/>
@@ -45978,10 +47388,10 @@
         <v>explicit</v>
       </c>
       <c r="E299" s="10" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="F299" s="11" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="G299" s="9"/>
       <c r="H299" s="9"/>
@@ -46102,13 +47512,13 @@
         <v>implicit</v>
       </c>
       <c r="E302" s="10" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="F302" s="11" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="G302" s="11" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="H302" s="9"/>
       <c r="I302" s="9"/>
@@ -46148,14 +47558,14 @@
         <v>external</v>
       </c>
       <c r="E303" s="10" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="F303" s="11" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="G303" s="9"/>
       <c r="H303" s="11" t="s">
-        <v>408</v>
+        <v>347</v>
       </c>
       <c r="I303" s="9"/>
       <c r="J303" s="9"/>
@@ -46234,13 +47644,13 @@
         <v>implicit</v>
       </c>
       <c r="E305" s="10" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="F305" s="11" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="G305" s="11" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="H305" s="9"/>
       <c r="I305" s="9"/>
@@ -46280,10 +47690,10 @@
         <v>external</v>
       </c>
       <c r="E306" s="10" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="F306" s="11" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="G306" s="9"/>
       <c r="H306" s="11" t="s">
@@ -46326,10 +47736,10 @@
         <v>external</v>
       </c>
       <c r="E307" s="10" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="F307" s="11" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="G307" s="9"/>
       <c r="H307" s="11" t="s">
@@ -46372,13 +47782,13 @@
         <v>implicit</v>
       </c>
       <c r="E308" s="10" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="F308" s="11" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="G308" s="11" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="H308" s="9"/>
       <c r="I308" s="9"/>
@@ -46419,16 +47829,16 @@
         <v>external</v>
       </c>
       <c r="E309" s="10" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="F309" s="11" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="G309" s="11" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="H309" s="11" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="I309" s="9"/>
       <c r="J309" s="9"/>
@@ -46467,10 +47877,10 @@
         <v>external</v>
       </c>
       <c r="E310" s="10" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="F310" s="11" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="G310" s="9"/>
       <c r="H310" s="11" t="s">
@@ -46513,10 +47923,10 @@
         <v>external</v>
       </c>
       <c r="E311" s="10" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="F311" s="11" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="G311" s="9"/>
       <c r="H311" s="11" t="s">
@@ -46559,13 +47969,13 @@
         <v>external</v>
       </c>
       <c r="E312" s="10" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="F312" s="11" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="G312" s="11" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="H312" s="11" t="s">
         <v>31</v>
@@ -46607,10 +48017,10 @@
         <v>external</v>
       </c>
       <c r="E313" s="10" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="F313" s="11" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="G313" s="9"/>
       <c r="H313" s="11" t="s">
@@ -46813,16 +48223,16 @@
         <v>external</v>
       </c>
       <c r="E318" s="10" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="F318" s="11" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="G318" s="11" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="H318" s="11" t="s">
-        <v>408</v>
+        <v>347</v>
       </c>
       <c r="I318" s="9"/>
       <c r="J318" s="9"/>
@@ -46982,16 +48392,16 @@
         <v>external</v>
       </c>
       <c r="E322" s="10" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="F322" s="11" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="G322" s="11" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="H322" s="11" t="s">
-        <v>408</v>
+        <v>347</v>
       </c>
       <c r="I322" s="9"/>
       <c r="J322" s="9"/>
@@ -47030,16 +48440,16 @@
         <v>external</v>
       </c>
       <c r="E323" s="10" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="F323" s="11" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="G323" s="11" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="H323" s="11" t="s">
-        <v>408</v>
+        <v>347</v>
       </c>
       <c r="I323" s="9"/>
       <c r="J323" s="9"/>
@@ -47117,9 +48527,15 @@
         <f t="array" ref="D325">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A324)-1, 23)+1, INT((ROW(A324)-1)/23)+1)</f>
         <v>implicit</v>
       </c>
-      <c r="E325" s="9"/>
-      <c r="F325" s="9"/>
-      <c r="G325" s="9"/>
+      <c r="E325" s="10" t="s">
+        <v>436</v>
+      </c>
+      <c r="F325" s="11" t="s">
+        <v>437</v>
+      </c>
+      <c r="G325" s="11" t="s">
+        <v>438</v>
+      </c>
       <c r="H325" s="9"/>
       <c r="I325" s="9"/>
       <c r="J325" s="9"/>
@@ -47197,8 +48613,12 @@
         <f t="array" ref="D327">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A326)-1, 23)+1, INT((ROW(A326)-1)/23)+1)</f>
         <v>explicit</v>
       </c>
-      <c r="E327" s="9"/>
-      <c r="F327" s="9"/>
+      <c r="E327" s="10" t="s">
+        <v>439</v>
+      </c>
+      <c r="F327" s="11" t="s">
+        <v>440</v>
+      </c>
       <c r="G327" s="9"/>
       <c r="H327" s="9"/>
       <c r="I327" s="9"/>
@@ -47237,9 +48657,15 @@
         <f t="array" ref="D328">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A327)-1, 23)+1, INT((ROW(A327)-1)/23)+1)</f>
         <v>implicit</v>
       </c>
-      <c r="E328" s="9"/>
-      <c r="F328" s="9"/>
-      <c r="G328" s="9"/>
+      <c r="E328" s="10" t="s">
+        <v>441</v>
+      </c>
+      <c r="F328" s="11" t="s">
+        <v>442</v>
+      </c>
+      <c r="G328" s="11" t="s">
+        <v>443</v>
+      </c>
       <c r="H328" s="9"/>
       <c r="I328" s="9"/>
       <c r="J328" s="9"/>
@@ -47277,9 +48703,15 @@
         <f t="array" ref="D329">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A328)-1, 23)+1, INT((ROW(A328)-1)/23)+1)</f>
         <v>implicit</v>
       </c>
-      <c r="E329" s="9"/>
-      <c r="F329" s="9"/>
-      <c r="G329" s="9"/>
+      <c r="E329" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="F329" s="11" t="s">
+        <v>445</v>
+      </c>
+      <c r="G329" s="11" t="s">
+        <v>446</v>
+      </c>
       <c r="H329" s="9"/>
       <c r="I329" s="9"/>
       <c r="J329" s="9"/>
@@ -47317,10 +48749,18 @@
         <f t="array" ref="D330">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A329)-1, 23)+1, INT((ROW(A329)-1)/23)+1)</f>
         <v>external</v>
       </c>
-      <c r="E330" s="9"/>
-      <c r="F330" s="9"/>
-      <c r="G330" s="9"/>
-      <c r="H330" s="9"/>
+      <c r="E330" s="10" t="s">
+        <v>447</v>
+      </c>
+      <c r="F330" s="11" t="s">
+        <v>448</v>
+      </c>
+      <c r="G330" s="11" t="s">
+        <v>449</v>
+      </c>
+      <c r="H330" s="11" t="s">
+        <v>205</v>
+      </c>
       <c r="I330" s="9"/>
       <c r="J330" s="9"/>
       <c r="K330" s="9"/>
@@ -47357,9 +48797,15 @@
         <f t="array" ref="D331">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A330)-1, 23)+1, INT((ROW(A330)-1)/23)+1)</f>
         <v>implicit</v>
       </c>
-      <c r="E331" s="9"/>
-      <c r="F331" s="9"/>
-      <c r="G331" s="9"/>
+      <c r="E331" s="10" t="s">
+        <v>450</v>
+      </c>
+      <c r="F331" s="11" t="s">
+        <v>451</v>
+      </c>
+      <c r="G331" s="11" t="s">
+        <v>452</v>
+      </c>
       <c r="H331" s="9"/>
       <c r="I331" s="9"/>
       <c r="J331" s="9"/>
@@ -47438,8 +48884,12 @@
         <f t="array" ref="D333">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A332)-1, 23)+1, INT((ROW(A332)-1)/23)+1)</f>
         <v>explicit</v>
       </c>
-      <c r="E333" s="9"/>
-      <c r="F333" s="9"/>
+      <c r="E333" s="10" t="s">
+        <v>453</v>
+      </c>
+      <c r="F333" s="11" t="s">
+        <v>454</v>
+      </c>
       <c r="G333" s="9"/>
       <c r="H333" s="9"/>
       <c r="I333" s="9"/>
@@ -47478,8 +48928,12 @@
         <f t="array" ref="D334">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A333)-1, 23)+1, INT((ROW(A333)-1)/23)+1)</f>
         <v>explicit</v>
       </c>
-      <c r="E334" s="9"/>
-      <c r="F334" s="9"/>
+      <c r="E334" s="10" t="s">
+        <v>455</v>
+      </c>
+      <c r="F334" s="11" t="s">
+        <v>456</v>
+      </c>
       <c r="G334" s="9"/>
       <c r="H334" s="9"/>
       <c r="I334" s="9"/>
@@ -47518,8 +48972,12 @@
         <f t="array" ref="D335">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A334)-1, 23)+1, INT((ROW(A334)-1)/23)+1)</f>
         <v>explicit</v>
       </c>
-      <c r="E335" s="9"/>
-      <c r="F335" s="9"/>
+      <c r="E335" s="10" t="s">
+        <v>457</v>
+      </c>
+      <c r="F335" s="11" t="s">
+        <v>458</v>
+      </c>
       <c r="G335" s="9"/>
       <c r="H335" s="9"/>
       <c r="I335" s="9"/>
@@ -47558,9 +49016,15 @@
         <f t="array" ref="D336">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A335)-1, 23)+1, INT((ROW(A335)-1)/23)+1)</f>
         <v>implicit</v>
       </c>
-      <c r="E336" s="9"/>
-      <c r="F336" s="9"/>
-      <c r="G336" s="9"/>
+      <c r="E336" s="10" t="s">
+        <v>459</v>
+      </c>
+      <c r="F336" s="11" t="s">
+        <v>460</v>
+      </c>
+      <c r="G336" s="11" t="s">
+        <v>461</v>
+      </c>
       <c r="H336" s="9"/>
       <c r="I336" s="9"/>
       <c r="J336" s="9"/>
@@ -47758,8 +49222,12 @@
         <f t="array" ref="D341">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A340)-1, 23)+1, INT((ROW(A340)-1)/23)+1)</f>
         <v>explicit</v>
       </c>
-      <c r="E341" s="9"/>
-      <c r="F341" s="9"/>
+      <c r="E341" s="10" t="s">
+        <v>462</v>
+      </c>
+      <c r="F341" s="11" t="s">
+        <v>463</v>
+      </c>
       <c r="G341" s="9"/>
       <c r="H341" s="9"/>
       <c r="I341" s="9"/>
@@ -47879,9 +49347,15 @@
         <f t="array" ref="D344">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A343)-1, 23)+1, INT((ROW(A343)-1)/23)+1)</f>
         <v>implicit</v>
       </c>
-      <c r="E344" s="9"/>
-      <c r="F344" s="9"/>
-      <c r="G344" s="9"/>
+      <c r="E344" s="10" t="s">
+        <v>464</v>
+      </c>
+      <c r="F344" s="11" t="s">
+        <v>465</v>
+      </c>
+      <c r="G344" s="11" t="s">
+        <v>466</v>
+      </c>
       <c r="H344" s="9"/>
       <c r="I344" s="9"/>
       <c r="J344" s="9"/>
@@ -47919,10 +49393,18 @@
         <f t="array" ref="D345">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A344)-1, 23)+1, INT((ROW(A344)-1)/23)+1)</f>
         <v>external</v>
       </c>
-      <c r="E345" s="9"/>
-      <c r="F345" s="9"/>
-      <c r="G345" s="9"/>
-      <c r="H345" s="9"/>
+      <c r="E345" s="10" t="s">
+        <v>467</v>
+      </c>
+      <c r="F345" s="11" t="s">
+        <v>468</v>
+      </c>
+      <c r="G345" s="11" t="s">
+        <v>469</v>
+      </c>
+      <c r="H345" s="11" t="s">
+        <v>470</v>
+      </c>
       <c r="I345" s="9"/>
       <c r="J345" s="9"/>
       <c r="K345" s="9"/>
@@ -47959,10 +49441,18 @@
         <f t="array" ref="D346">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A345)-1, 23)+1, INT((ROW(A345)-1)/23)+1)</f>
         <v>external</v>
       </c>
-      <c r="E346" s="9"/>
-      <c r="F346" s="9"/>
-      <c r="G346" s="9"/>
-      <c r="H346" s="9"/>
+      <c r="E346" s="10" t="s">
+        <v>471</v>
+      </c>
+      <c r="F346" s="11" t="s">
+        <v>472</v>
+      </c>
+      <c r="G346" s="11" t="s">
+        <v>473</v>
+      </c>
+      <c r="H346" s="11" t="s">
+        <v>474</v>
+      </c>
       <c r="I346" s="9"/>
       <c r="J346" s="9"/>
       <c r="K346" s="9"/>
@@ -48039,9 +49529,15 @@
         <f t="array" ref="D348">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A347)-1, 23)+1, INT((ROW(A347)-1)/23)+1)</f>
         <v>implicit</v>
       </c>
-      <c r="E348" s="9"/>
-      <c r="F348" s="9"/>
-      <c r="G348" s="9"/>
+      <c r="E348" s="10" t="s">
+        <v>475</v>
+      </c>
+      <c r="F348" s="11" t="s">
+        <v>476</v>
+      </c>
+      <c r="G348" s="11" t="s">
+        <v>477</v>
+      </c>
       <c r="H348" s="9"/>
       <c r="I348" s="9"/>
       <c r="J348" s="9"/>
@@ -48159,9 +49655,15 @@
         <f t="array" ref="D351">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A350)-1, 23)+1, INT((ROW(A350)-1)/23)+1)</f>
         <v>implicit</v>
       </c>
-      <c r="E351" s="9"/>
-      <c r="F351" s="9"/>
-      <c r="G351" s="9"/>
+      <c r="E351" s="10" t="s">
+        <v>478</v>
+      </c>
+      <c r="F351" s="11" t="s">
+        <v>476</v>
+      </c>
+      <c r="G351" s="11" t="s">
+        <v>479</v>
+      </c>
       <c r="H351" s="9"/>
       <c r="I351" s="9"/>
       <c r="J351" s="9"/>
@@ -48199,9 +49701,15 @@
         <f t="array" ref="D352">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A351)-1, 23)+1, INT((ROW(A351)-1)/23)+1)</f>
         <v>implicit</v>
       </c>
-      <c r="E352" s="9"/>
-      <c r="F352" s="9"/>
-      <c r="G352" s="9"/>
+      <c r="E352" s="10" t="s">
+        <v>480</v>
+      </c>
+      <c r="F352" s="11" t="s">
+        <v>481</v>
+      </c>
+      <c r="G352" s="11" t="s">
+        <v>482</v>
+      </c>
       <c r="H352" s="9"/>
       <c r="I352" s="9"/>
       <c r="J352" s="9"/>
@@ -48239,10 +49747,16 @@
         <f t="array" ref="D353">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A352)-1, 23)+1, INT((ROW(A352)-1)/23)+1)</f>
         <v>external</v>
       </c>
-      <c r="E353" s="9"/>
-      <c r="F353" s="9"/>
+      <c r="E353" s="10" t="s">
+        <v>483</v>
+      </c>
+      <c r="F353" s="11" t="s">
+        <v>484</v>
+      </c>
       <c r="G353" s="9"/>
-      <c r="H353" s="9"/>
+      <c r="H353" s="11" t="s">
+        <v>205</v>
+      </c>
       <c r="I353" s="9"/>
       <c r="J353" s="9"/>
       <c r="K353" s="9"/>
@@ -48320,9 +49834,15 @@
         <f t="array" ref="D355">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A354)-1, 23)+1, INT((ROW(A354)-1)/23)+1)</f>
         <v>implicit</v>
       </c>
-      <c r="E355" s="9"/>
-      <c r="F355" s="9"/>
-      <c r="G355" s="9"/>
+      <c r="E355" s="10" t="s">
+        <v>485</v>
+      </c>
+      <c r="F355" s="11" t="s">
+        <v>486</v>
+      </c>
+      <c r="G355" s="11" t="s">
+        <v>487</v>
+      </c>
       <c r="H355" s="9"/>
       <c r="I355" s="9"/>
       <c r="J355" s="9"/>
@@ -48360,8 +49880,12 @@
         <f t="array" ref="D356">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A355)-1, 23)+1, INT((ROW(A355)-1)/23)+1)</f>
         <v>explicit</v>
       </c>
-      <c r="E356" s="9"/>
-      <c r="F356" s="9"/>
+      <c r="E356" s="15" t="s">
+        <v>488</v>
+      </c>
+      <c r="F356" s="11" t="s">
+        <v>489</v>
+      </c>
       <c r="G356" s="9"/>
       <c r="H356" s="9"/>
       <c r="I356" s="9"/>
@@ -48400,9 +49924,15 @@
         <f t="array" ref="D357">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A356)-1, 23)+1, INT((ROW(A356)-1)/23)+1)</f>
         <v>implicit</v>
       </c>
-      <c r="E357" s="9"/>
-      <c r="F357" s="9"/>
-      <c r="G357" s="9"/>
+      <c r="E357" s="10" t="s">
+        <v>490</v>
+      </c>
+      <c r="F357" s="11" t="s">
+        <v>491</v>
+      </c>
+      <c r="G357" s="11" t="s">
+        <v>492</v>
+      </c>
       <c r="H357" s="9"/>
       <c r="I357" s="9"/>
       <c r="J357" s="9"/>
@@ -48440,10 +49970,16 @@
         <f t="array" ref="D358">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A357)-1, 23)+1, INT((ROW(A357)-1)/23)+1)</f>
         <v>external</v>
       </c>
-      <c r="E358" s="9"/>
-      <c r="F358" s="9"/>
+      <c r="E358" s="15" t="s">
+        <v>493</v>
+      </c>
+      <c r="F358" s="11" t="s">
+        <v>494</v>
+      </c>
       <c r="G358" s="9"/>
-      <c r="H358" s="9"/>
+      <c r="H358" s="11" t="s">
+        <v>495</v>
+      </c>
       <c r="I358" s="9"/>
       <c r="J358" s="9"/>
       <c r="K358" s="9"/>
@@ -48480,9 +50016,15 @@
         <f t="array" ref="D359">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A358)-1, 23)+1, INT((ROW(A358)-1)/23)+1)</f>
         <v>implicit</v>
       </c>
-      <c r="E359" s="9"/>
-      <c r="F359" s="9"/>
-      <c r="G359" s="9"/>
+      <c r="E359" s="15" t="s">
+        <v>496</v>
+      </c>
+      <c r="F359" s="11" t="s">
+        <v>497</v>
+      </c>
+      <c r="G359" s="11" t="s">
+        <v>498</v>
+      </c>
       <c r="H359" s="9"/>
       <c r="I359" s="9"/>
       <c r="J359" s="9"/>
@@ -48680,10 +50222,16 @@
         <f t="array" ref="D364">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A363)-1, 23)+1, INT((ROW(A363)-1)/23)+1)</f>
         <v>external</v>
       </c>
-      <c r="E364" s="9"/>
-      <c r="F364" s="9"/>
+      <c r="E364" s="10" t="s">
+        <v>499</v>
+      </c>
+      <c r="F364" s="11" t="s">
+        <v>500</v>
+      </c>
       <c r="G364" s="9"/>
-      <c r="H364" s="9"/>
+      <c r="H364" s="11" t="s">
+        <v>501</v>
+      </c>
       <c r="I364" s="9"/>
       <c r="J364" s="9"/>
       <c r="K364" s="9"/>
@@ -48841,10 +50389,16 @@
         <f t="array" ref="D368">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A367)-1, 23)+1, INT((ROW(A367)-1)/23)+1)</f>
         <v>external</v>
       </c>
-      <c r="E368" s="9"/>
-      <c r="F368" s="9"/>
+      <c r="E368" s="15" t="s">
+        <v>502</v>
+      </c>
+      <c r="F368" s="11" t="s">
+        <v>503</v>
+      </c>
       <c r="G368" s="9"/>
-      <c r="H368" s="9"/>
+      <c r="H368" s="11" t="s">
+        <v>504</v>
+      </c>
       <c r="I368" s="9"/>
       <c r="J368" s="9"/>
       <c r="K368" s="9"/>
@@ -48881,10 +50435,18 @@
         <f t="array" ref="D369">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A368)-1, 23)+1, INT((ROW(A368)-1)/23)+1)</f>
         <v>external</v>
       </c>
-      <c r="E369" s="9"/>
-      <c r="F369" s="9"/>
-      <c r="G369" s="9"/>
-      <c r="H369" s="9"/>
+      <c r="E369" s="10" t="s">
+        <v>505</v>
+      </c>
+      <c r="F369" s="11" t="s">
+        <v>506</v>
+      </c>
+      <c r="G369" s="11" t="s">
+        <v>507</v>
+      </c>
+      <c r="H369" s="11" t="s">
+        <v>176</v>
+      </c>
       <c r="I369" s="9"/>
       <c r="J369" s="9"/>
       <c r="K369" s="9"/>
@@ -48945,13 +50507,31 @@
       <c r="Z370" s="9"/>
     </row>
     <row r="371">
-      <c r="A371" s="9"/>
-      <c r="B371" s="9"/>
-      <c r="C371" s="9"/>
-      <c r="D371" s="9"/>
-      <c r="E371" s="9"/>
-      <c r="F371" s="9"/>
-      <c r="G371" s="9"/>
+      <c r="A371" s="5" t="str">
+        <f t="array" ref="A371">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A370)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B371" s="5" t="str">
+        <f t="array" ref="B371">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B370)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C371" s="5" t="str">
+        <f t="array" ref="C371">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A370)-1, 23)+1)</f>
+        <v>Experiment Manager</v>
+      </c>
+      <c r="D371" s="5" t="str">
+        <f t="array" ref="D371">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A370)-1, 23)+1, INT((ROW(A370)-1)/23)+1)</f>
+        <v>implicit</v>
+      </c>
+      <c r="E371" s="10" t="s">
+        <v>508</v>
+      </c>
+      <c r="F371" s="11" t="s">
+        <v>509</v>
+      </c>
+      <c r="G371" s="11" t="s">
+        <v>510</v>
+      </c>
       <c r="H371" s="9"/>
       <c r="I371" s="9"/>
       <c r="J371" s="9"/>
@@ -48973,10 +50553,22 @@
       <c r="Z371" s="9"/>
     </row>
     <row r="372">
-      <c r="A372" s="9"/>
-      <c r="B372" s="9"/>
-      <c r="C372" s="9"/>
-      <c r="D372" s="9"/>
+      <c r="A372" s="5" t="str">
+        <f t="array" ref="A372">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A371)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B372" s="5" t="str">
+        <f t="array" ref="B372">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B371)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C372" s="5" t="str">
+        <f t="array" ref="C372">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A371)-1, 23)+1)</f>
+        <v>Hyperparameter Tuner</v>
+      </c>
+      <c r="D372" s="5" t="str">
+        <f t="array" ref="D372">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A371)-1, 23)+1, INT((ROW(A371)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E372" s="9"/>
       <c r="F372" s="9"/>
       <c r="G372" s="9"/>
@@ -49001,10 +50593,22 @@
       <c r="Z372" s="9"/>
     </row>
     <row r="373">
-      <c r="A373" s="9"/>
-      <c r="B373" s="9"/>
-      <c r="C373" s="9"/>
-      <c r="D373" s="9"/>
+      <c r="A373" s="5" t="str">
+        <f t="array" ref="A373">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A372)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B373" s="5" t="str">
+        <f t="array" ref="B373">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B372)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C373" s="5" t="str">
+        <f t="array" ref="C373">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A372)-1, 23)+1)</f>
+        <v>Benchmark Manager</v>
+      </c>
+      <c r="D373" s="5" t="str">
+        <f t="array" ref="D373">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A372)-1, 23)+1, INT((ROW(A372)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E373" s="9"/>
       <c r="F373" s="9"/>
       <c r="G373" s="9"/>
@@ -49029,13 +50633,31 @@
       <c r="Z373" s="9"/>
     </row>
     <row r="374">
-      <c r="A374" s="9"/>
-      <c r="B374" s="9"/>
-      <c r="C374" s="9"/>
-      <c r="D374" s="9"/>
-      <c r="E374" s="9"/>
-      <c r="F374" s="9"/>
-      <c r="G374" s="9"/>
+      <c r="A374" s="5" t="str">
+        <f t="array" ref="A374">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A373)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B374" s="5" t="str">
+        <f t="array" ref="B374">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B373)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C374" s="5" t="str">
+        <f t="array" ref="C374">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A373)-1, 23)+1)</f>
+        <v>Framework Orchestrator</v>
+      </c>
+      <c r="D374" s="5" t="str">
+        <f t="array" ref="D374">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A373)-1, 23)+1, INT((ROW(A373)-1)/23)+1)</f>
+        <v>implicit</v>
+      </c>
+      <c r="E374" s="10" t="s">
+        <v>511</v>
+      </c>
+      <c r="F374" s="11" t="s">
+        <v>509</v>
+      </c>
+      <c r="G374" s="11" t="s">
+        <v>512</v>
+      </c>
       <c r="H374" s="9"/>
       <c r="I374" s="9"/>
       <c r="J374" s="9"/>
@@ -49057,13 +50679,31 @@
       <c r="Z374" s="9"/>
     </row>
     <row r="375">
-      <c r="A375" s="9"/>
-      <c r="B375" s="9"/>
-      <c r="C375" s="9"/>
-      <c r="D375" s="9"/>
-      <c r="E375" s="9"/>
-      <c r="F375" s="9"/>
-      <c r="G375" s="9"/>
+      <c r="A375" s="5" t="str">
+        <f t="array" ref="A375">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A374)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B375" s="5" t="str">
+        <f t="array" ref="B375">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B374)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C375" s="5" t="str">
+        <f t="array" ref="C375">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A374)-1, 23)+1)</f>
+        <v>Lifecycle Manager</v>
+      </c>
+      <c r="D375" s="5" t="str">
+        <f t="array" ref="D375">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A374)-1, 23)+1, INT((ROW(A374)-1)/23)+1)</f>
+        <v>implicit</v>
+      </c>
+      <c r="E375" s="10" t="s">
+        <v>513</v>
+      </c>
+      <c r="F375" s="11" t="s">
+        <v>514</v>
+      </c>
+      <c r="G375" s="11" t="s">
+        <v>515</v>
+      </c>
       <c r="H375" s="9"/>
       <c r="I375" s="9"/>
       <c r="J375" s="9"/>
@@ -49085,14 +50725,32 @@
       <c r="Z375" s="9"/>
     </row>
     <row r="376">
-      <c r="A376" s="9"/>
-      <c r="B376" s="9"/>
-      <c r="C376" s="9"/>
-      <c r="D376" s="9"/>
-      <c r="E376" s="9"/>
-      <c r="F376" s="9"/>
+      <c r="A376" s="5" t="str">
+        <f t="array" ref="A376">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A375)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B376" s="5" t="str">
+        <f t="array" ref="B376">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B375)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C376" s="5" t="str">
+        <f t="array" ref="C376">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A375)-1, 23)+1)</f>
+        <v>Configuration Manager</v>
+      </c>
+      <c r="D376" s="5" t="str">
+        <f t="array" ref="D376">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A375)-1, 23)+1, INT((ROW(A375)-1)/23)+1)</f>
+        <v>external</v>
+      </c>
+      <c r="E376" s="10" t="s">
+        <v>516</v>
+      </c>
+      <c r="F376" s="11" t="s">
+        <v>517</v>
+      </c>
       <c r="G376" s="9"/>
-      <c r="H376" s="9"/>
+      <c r="H376" s="11" t="s">
+        <v>518</v>
+      </c>
       <c r="I376" s="9"/>
       <c r="J376" s="9"/>
       <c r="K376" s="9"/>
@@ -49113,10 +50771,22 @@
       <c r="Z376" s="9"/>
     </row>
     <row r="377">
-      <c r="A377" s="9"/>
-      <c r="B377" s="9"/>
-      <c r="C377" s="9"/>
-      <c r="D377" s="9"/>
+      <c r="A377" s="5" t="str">
+        <f t="array" ref="A377">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A376)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B377" s="5" t="str">
+        <f t="array" ref="B377">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B376)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C377" s="5" t="str">
+        <f t="array" ref="C377">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A376)-1, 23)+1)</f>
+        <v>Multi-Agent Coordinator</v>
+      </c>
+      <c r="D377" s="5" t="str">
+        <f t="array" ref="D377">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A376)-1, 23)+1, INT((ROW(A376)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E377" s="9"/>
       <c r="F377" s="9"/>
       <c r="G377" s="9"/>
@@ -49141,10 +50811,23 @@
       <c r="Z377" s="9"/>
     </row>
     <row r="378">
-      <c r="A378" s="9"/>
-      <c r="B378" s="9"/>
-      <c r="C378" s="9"/>
-      <c r="D378" s="9"/>
+      <c r="A378" s="5" t="str">
+        <f t="array" ref="A378">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A377)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B378" s="5" t="str">
+        <f t="array" ref="B378">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B377)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C378" s="5" t="str">
+        <f t="array" ref="C378">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A377)-1, 23)+1)</f>
+        <v>Distributed Execution 
+Coordinator</v>
+      </c>
+      <c r="D378" s="5" t="str">
+        <f t="array" ref="D378">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A377)-1, 23)+1, INT((ROW(A377)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E378" s="9"/>
       <c r="F378" s="9"/>
       <c r="G378" s="9"/>
@@ -49169,13 +50852,31 @@
       <c r="Z378" s="9"/>
     </row>
     <row r="379">
-      <c r="A379" s="9"/>
-      <c r="B379" s="9"/>
-      <c r="C379" s="9"/>
-      <c r="D379" s="9"/>
-      <c r="E379" s="9"/>
-      <c r="F379" s="9"/>
-      <c r="G379" s="9"/>
+      <c r="A379" s="5" t="str">
+        <f t="array" ref="A379">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A378)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B379" s="5" t="str">
+        <f t="array" ref="B379">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B378)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C379" s="5" t="str">
+        <f t="array" ref="C379">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A378)-1, 23)+1)</f>
+        <v>Agent</v>
+      </c>
+      <c r="D379" s="5" t="str">
+        <f t="array" ref="D379">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A378)-1, 23)+1, INT((ROW(A378)-1)/23)+1)</f>
+        <v>explicit</v>
+      </c>
+      <c r="E379" s="15" t="s">
+        <v>519</v>
+      </c>
+      <c r="F379" s="11" t="s">
+        <v>520</v>
+      </c>
+      <c r="G379" s="11" t="s">
+        <v>521</v>
+      </c>
       <c r="H379" s="9"/>
       <c r="I379" s="9"/>
       <c r="J379" s="9"/>
@@ -49197,13 +50898,31 @@
       <c r="Z379" s="9"/>
     </row>
     <row r="380">
-      <c r="A380" s="9"/>
-      <c r="B380" s="9"/>
-      <c r="C380" s="9"/>
-      <c r="D380" s="9"/>
-      <c r="E380" s="9"/>
-      <c r="F380" s="9"/>
-      <c r="G380" s="9"/>
+      <c r="A380" s="5" t="str">
+        <f t="array" ref="A380">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A379)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B380" s="5" t="str">
+        <f t="array" ref="B380">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B379)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C380" s="5" t="str">
+        <f t="array" ref="C380">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A379)-1, 23)+1)</f>
+        <v>Function Approximator</v>
+      </c>
+      <c r="D380" s="5" t="str">
+        <f t="array" ref="D380">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A379)-1, 23)+1, INT((ROW(A379)-1)/23)+1)</f>
+        <v>implicit</v>
+      </c>
+      <c r="E380" s="10" t="s">
+        <v>522</v>
+      </c>
+      <c r="F380" s="11" t="s">
+        <v>523</v>
+      </c>
+      <c r="G380" s="11" t="s">
+        <v>524</v>
+      </c>
       <c r="H380" s="9"/>
       <c r="I380" s="9"/>
       <c r="J380" s="9"/>
@@ -49225,12 +50944,28 @@
       <c r="Z380" s="9"/>
     </row>
     <row r="381">
-      <c r="A381" s="9"/>
-      <c r="B381" s="9"/>
-      <c r="C381" s="9"/>
-      <c r="D381" s="9"/>
-      <c r="E381" s="9"/>
-      <c r="F381" s="9"/>
+      <c r="A381" s="5" t="str">
+        <f t="array" ref="A381">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A380)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B381" s="5" t="str">
+        <f t="array" ref="B381">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B380)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C381" s="5" t="str">
+        <f t="array" ref="C381">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A380)-1, 23)+1)</f>
+        <v>Buffer</v>
+      </c>
+      <c r="D381" s="5" t="str">
+        <f t="array" ref="D381">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A380)-1, 23)+1, INT((ROW(A380)-1)/23)+1)</f>
+        <v>explicit</v>
+      </c>
+      <c r="E381" s="10" t="s">
+        <v>525</v>
+      </c>
+      <c r="F381" s="11" t="s">
+        <v>526</v>
+      </c>
       <c r="G381" s="9"/>
       <c r="H381" s="9"/>
       <c r="I381" s="9"/>
@@ -49253,13 +50988,31 @@
       <c r="Z381" s="9"/>
     </row>
     <row r="382">
-      <c r="A382" s="9"/>
-      <c r="B382" s="9"/>
-      <c r="C382" s="9"/>
-      <c r="D382" s="9"/>
-      <c r="E382" s="9"/>
-      <c r="F382" s="9"/>
-      <c r="G382" s="9"/>
+      <c r="A382" s="5" t="str">
+        <f t="array" ref="A382">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A381)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B382" s="5" t="str">
+        <f t="array" ref="B382">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B381)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C382" s="5" t="str">
+        <f t="array" ref="C382">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A381)-1, 23)+1)</f>
+        <v>Learner</v>
+      </c>
+      <c r="D382" s="5" t="str">
+        <f t="array" ref="D382">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A381)-1, 23)+1, INT((ROW(A381)-1)/23)+1)</f>
+        <v>implicit</v>
+      </c>
+      <c r="E382" s="10" t="s">
+        <v>527</v>
+      </c>
+      <c r="F382" s="11" t="s">
+        <v>528</v>
+      </c>
+      <c r="G382" s="11" t="s">
+        <v>529</v>
+      </c>
       <c r="H382" s="9"/>
       <c r="I382" s="9"/>
       <c r="J382" s="9"/>
@@ -49281,10 +51034,22 @@
       <c r="Z382" s="9"/>
     </row>
     <row r="383">
-      <c r="A383" s="9"/>
-      <c r="B383" s="9"/>
-      <c r="C383" s="9"/>
-      <c r="D383" s="9"/>
+      <c r="A383" s="5" t="str">
+        <f t="array" ref="A383">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A382)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B383" s="5" t="str">
+        <f t="array" ref="B383">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B382)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C383" s="5" t="str">
+        <f t="array" ref="C383">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A382)-1, 23)+1)</f>
+        <v>Environment</v>
+      </c>
+      <c r="D383" s="5" t="str">
+        <f t="array" ref="D383">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A382)-1, 23)+1, INT((ROW(A382)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E383" s="9"/>
       <c r="F383" s="9"/>
       <c r="G383" s="9"/>
@@ -49309,10 +51074,22 @@
       <c r="Z383" s="9"/>
     </row>
     <row r="384">
-      <c r="A384" s="9"/>
-      <c r="B384" s="9"/>
-      <c r="C384" s="9"/>
-      <c r="D384" s="9"/>
+      <c r="A384" s="5" t="str">
+        <f t="array" ref="A384">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A383)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B384" s="5" t="str">
+        <f t="array" ref="B384">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B383)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C384" s="5" t="str">
+        <f t="array" ref="C384">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A383)-1, 23)+1)</f>
+        <v>Environment Core</v>
+      </c>
+      <c r="D384" s="5" t="str">
+        <f t="array" ref="D384">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A383)-1, 23)+1, INT((ROW(A383)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E384" s="9"/>
       <c r="F384" s="9"/>
       <c r="G384" s="9"/>
@@ -49337,10 +51114,22 @@
       <c r="Z384" s="9"/>
     </row>
     <row r="385">
-      <c r="A385" s="9"/>
-      <c r="B385" s="9"/>
-      <c r="C385" s="9"/>
-      <c r="D385" s="9"/>
+      <c r="A385" s="5" t="str">
+        <f t="array" ref="A385">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A384)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B385" s="5" t="str">
+        <f t="array" ref="B385">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B384)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C385" s="5" t="str">
+        <f t="array" ref="C385">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A384)-1, 23)+1)</f>
+        <v>Simulator</v>
+      </c>
+      <c r="D385" s="5" t="str">
+        <f t="array" ref="D385">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A384)-1, 23)+1, INT((ROW(A384)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E385" s="9"/>
       <c r="F385" s="9"/>
       <c r="G385" s="9"/>
@@ -49365,10 +51154,22 @@
       <c r="Z385" s="9"/>
     </row>
     <row r="386">
-      <c r="A386" s="9"/>
-      <c r="B386" s="9"/>
-      <c r="C386" s="9"/>
-      <c r="D386" s="9"/>
+      <c r="A386" s="5" t="str">
+        <f t="array" ref="A386">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A385)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B386" s="5" t="str">
+        <f t="array" ref="B386">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B385)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C386" s="5" t="str">
+        <f t="array" ref="C386">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A385)-1, 23)+1)</f>
+        <v>Simulator Adapter</v>
+      </c>
+      <c r="D386" s="5" t="str">
+        <f t="array" ref="D386">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A385)-1, 23)+1, INT((ROW(A385)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E386" s="9"/>
       <c r="F386" s="9"/>
       <c r="G386" s="9"/>
@@ -49393,12 +51194,28 @@
       <c r="Z386" s="9"/>
     </row>
     <row r="387">
-      <c r="A387" s="9"/>
-      <c r="B387" s="9"/>
-      <c r="C387" s="9"/>
-      <c r="D387" s="9"/>
-      <c r="E387" s="9"/>
-      <c r="F387" s="9"/>
+      <c r="A387" s="5" t="str">
+        <f t="array" ref="A387">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A386)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B387" s="5" t="str">
+        <f t="array" ref="B387">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B386)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C387" s="5" t="str">
+        <f t="array" ref="C387">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A386)-1, 23)+1)</f>
+        <v>Checkpoint Manager</v>
+      </c>
+      <c r="D387" s="5" t="str">
+        <f t="array" ref="D387">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A386)-1, 23)+1, INT((ROW(A386)-1)/23)+1)</f>
+        <v>explicit</v>
+      </c>
+      <c r="E387" s="10" t="s">
+        <v>530</v>
+      </c>
+      <c r="F387" s="11" t="s">
+        <v>531</v>
+      </c>
       <c r="G387" s="9"/>
       <c r="H387" s="9"/>
       <c r="I387" s="9"/>
@@ -49421,10 +51238,23 @@
       <c r="Z387" s="9"/>
     </row>
     <row r="388">
-      <c r="A388" s="9"/>
-      <c r="B388" s="9"/>
-      <c r="C388" s="9"/>
-      <c r="D388" s="9"/>
+      <c r="A388" s="5" t="str">
+        <f t="array" ref="A388">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A387)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B388" s="5" t="str">
+        <f t="array" ref="B388">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B387)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C388" s="5" t="str">
+        <f t="array" ref="C388">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A387)-1, 23)+1)</f>
+        <v>Environment Parameter 
+Manager</v>
+      </c>
+      <c r="D388" s="5" t="str">
+        <f t="array" ref="D388">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A387)-1, 23)+1, INT((ROW(A387)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E388" s="9"/>
       <c r="F388" s="9"/>
       <c r="G388" s="9"/>
@@ -49449,10 +51279,22 @@
       <c r="Z388" s="9"/>
     </row>
     <row r="389">
-      <c r="A389" s="9"/>
-      <c r="B389" s="9"/>
-      <c r="C389" s="9"/>
-      <c r="D389" s="9"/>
+      <c r="A389" s="5" t="str">
+        <f t="array" ref="A389">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A388)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B389" s="5" t="str">
+        <f t="array" ref="B389">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B388)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C389" s="5" t="str">
+        <f t="array" ref="C389">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A388)-1, 23)+1)</f>
+        <v>Renderer</v>
+      </c>
+      <c r="D389" s="5" t="str">
+        <f t="array" ref="D389">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A388)-1, 23)+1, INT((ROW(A388)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E389" s="9"/>
       <c r="F389" s="9"/>
       <c r="G389" s="9"/>
@@ -49477,13 +51319,31 @@
       <c r="Z389" s="9"/>
     </row>
     <row r="390">
-      <c r="A390" s="9"/>
-      <c r="B390" s="9"/>
-      <c r="C390" s="9"/>
-      <c r="D390" s="9"/>
-      <c r="E390" s="9"/>
-      <c r="F390" s="9"/>
-      <c r="G390" s="9"/>
+      <c r="A390" s="5" t="str">
+        <f t="array" ref="A390">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A389)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B390" s="5" t="str">
+        <f t="array" ref="B390">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B389)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C390" s="5" t="str">
+        <f t="array" ref="C390">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A389)-1, 23)+1)</f>
+        <v>Recorder</v>
+      </c>
+      <c r="D390" s="5" t="str">
+        <f t="array" ref="D390">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A389)-1, 23)+1, INT((ROW(A389)-1)/23)+1)</f>
+        <v>explicit</v>
+      </c>
+      <c r="E390" s="10" t="s">
+        <v>532</v>
+      </c>
+      <c r="F390" s="11" t="s">
+        <v>533</v>
+      </c>
+      <c r="G390" s="11" t="s">
+        <v>534</v>
+      </c>
       <c r="H390" s="9"/>
       <c r="I390" s="9"/>
       <c r="J390" s="9"/>
@@ -49505,12 +51365,28 @@
       <c r="Z390" s="9"/>
     </row>
     <row r="391">
-      <c r="A391" s="9"/>
-      <c r="B391" s="9"/>
-      <c r="C391" s="9"/>
-      <c r="D391" s="9"/>
-      <c r="E391" s="9"/>
-      <c r="F391" s="9"/>
+      <c r="A391" s="5" t="str">
+        <f t="array" ref="A391">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A390)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B391" s="5" t="str">
+        <f t="array" ref="B391">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B390)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C391" s="5" t="str">
+        <f t="array" ref="C391">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A390)-1, 23)+1)</f>
+        <v>Logger</v>
+      </c>
+      <c r="D391" s="5" t="str">
+        <f t="array" ref="D391">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A390)-1, 23)+1, INT((ROW(A390)-1)/23)+1)</f>
+        <v>explicit</v>
+      </c>
+      <c r="E391" s="10" t="s">
+        <v>535</v>
+      </c>
+      <c r="F391" s="11" t="s">
+        <v>536</v>
+      </c>
       <c r="G391" s="9"/>
       <c r="H391" s="9"/>
       <c r="I391" s="9"/>
@@ -49533,14 +51409,32 @@
       <c r="Z391" s="9"/>
     </row>
     <row r="392">
-      <c r="A392" s="9"/>
-      <c r="B392" s="9"/>
-      <c r="C392" s="9"/>
-      <c r="D392" s="9"/>
-      <c r="E392" s="9"/>
-      <c r="F392" s="9"/>
+      <c r="A392" s="5" t="str">
+        <f t="array" ref="A392">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A391)-1)/23)+1)</f>
+        <v>F17</v>
+      </c>
+      <c r="B392" s="5" t="str">
+        <f t="array" ref="B392">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B391)-1)/23)+1)</f>
+        <v>Dopamine</v>
+      </c>
+      <c r="C392" s="5" t="str">
+        <f t="array" ref="C392">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A391)-1, 23)+1)</f>
+        <v>Reporter</v>
+      </c>
+      <c r="D392" s="5" t="str">
+        <f t="array" ref="D392">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A391)-1, 23)+1, INT((ROW(A391)-1)/23)+1)</f>
+        <v>external</v>
+      </c>
+      <c r="E392" s="10" t="s">
+        <v>537</v>
+      </c>
+      <c r="F392" s="11" t="s">
+        <v>538</v>
+      </c>
       <c r="G392" s="9"/>
-      <c r="H392" s="9"/>
+      <c r="H392" s="11" t="s">
+        <v>176</v>
+      </c>
       <c r="I392" s="9"/>
       <c r="J392" s="9"/>
       <c r="K392" s="9"/>
@@ -49561,10 +51455,22 @@
       <c r="Z392" s="9"/>
     </row>
     <row r="393">
-      <c r="A393" s="9"/>
-      <c r="B393" s="9"/>
-      <c r="C393" s="9"/>
-      <c r="D393" s="9"/>
+      <c r="A393" s="5" t="str">
+        <f t="array" ref="A393">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A392)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B393" s="5" t="str">
+        <f t="array" ref="B393">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B392)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C393" s="5" t="str">
+        <f t="array" ref="C393">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A392)-1, 23)+1)</f>
+        <v>Experiment Orchestrator</v>
+      </c>
+      <c r="D393" s="5" t="str">
+        <f t="array" ref="D393">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A392)-1, 23)+1, INT((ROW(A392)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E393" s="9"/>
       <c r="F393" s="9"/>
       <c r="G393" s="9"/>
@@ -49589,13 +51495,31 @@
       <c r="Z393" s="9"/>
     </row>
     <row r="394">
-      <c r="A394" s="9"/>
-      <c r="B394" s="9"/>
-      <c r="C394" s="9"/>
-      <c r="D394" s="9"/>
-      <c r="E394" s="9"/>
-      <c r="F394" s="9"/>
-      <c r="G394" s="9"/>
+      <c r="A394" s="5" t="str">
+        <f t="array" ref="A394">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A393)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B394" s="5" t="str">
+        <f t="array" ref="B394">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B393)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C394" s="5" t="str">
+        <f t="array" ref="C394">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A393)-1, 23)+1)</f>
+        <v>Experiment Manager</v>
+      </c>
+      <c r="D394" s="5" t="str">
+        <f t="array" ref="D394">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A393)-1, 23)+1, INT((ROW(A393)-1)/23)+1)</f>
+        <v>explicit</v>
+      </c>
+      <c r="E394" s="10" t="s">
+        <v>539</v>
+      </c>
+      <c r="F394" s="11" t="s">
+        <v>540</v>
+      </c>
+      <c r="G394" s="11" t="s">
+        <v>541</v>
+      </c>
       <c r="H394" s="9"/>
       <c r="I394" s="9"/>
       <c r="J394" s="9"/>
@@ -49617,10 +51541,22 @@
       <c r="Z394" s="9"/>
     </row>
     <row r="395">
-      <c r="A395" s="9"/>
-      <c r="B395" s="9"/>
-      <c r="C395" s="9"/>
-      <c r="D395" s="9"/>
+      <c r="A395" s="5" t="str">
+        <f t="array" ref="A395">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A394)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B395" s="5" t="str">
+        <f t="array" ref="B395">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B394)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C395" s="5" t="str">
+        <f t="array" ref="C395">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A394)-1, 23)+1)</f>
+        <v>Hyperparameter Tuner</v>
+      </c>
+      <c r="D395" s="5" t="str">
+        <f t="array" ref="D395">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A394)-1, 23)+1, INT((ROW(A394)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E395" s="9"/>
       <c r="F395" s="9"/>
       <c r="G395" s="9"/>
@@ -49645,10 +51581,22 @@
       <c r="Z395" s="9"/>
     </row>
     <row r="396">
-      <c r="A396" s="9"/>
-      <c r="B396" s="9"/>
-      <c r="C396" s="9"/>
-      <c r="D396" s="9"/>
+      <c r="A396" s="5" t="str">
+        <f t="array" ref="A396">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A395)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B396" s="5" t="str">
+        <f t="array" ref="B396">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B395)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C396" s="5" t="str">
+        <f t="array" ref="C396">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A395)-1, 23)+1)</f>
+        <v>Benchmark Manager</v>
+      </c>
+      <c r="D396" s="5" t="str">
+        <f t="array" ref="D396">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A395)-1, 23)+1, INT((ROW(A395)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E396" s="9"/>
       <c r="F396" s="9"/>
       <c r="G396" s="9"/>
@@ -49673,13 +51621,31 @@
       <c r="Z396" s="9"/>
     </row>
     <row r="397">
-      <c r="A397" s="9"/>
-      <c r="B397" s="9"/>
-      <c r="C397" s="9"/>
-      <c r="D397" s="9"/>
-      <c r="E397" s="9"/>
-      <c r="F397" s="9"/>
-      <c r="G397" s="9"/>
+      <c r="A397" s="5" t="str">
+        <f t="array" ref="A397">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A396)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B397" s="5" t="str">
+        <f t="array" ref="B397">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B396)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C397" s="5" t="str">
+        <f t="array" ref="C397">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A396)-1, 23)+1)</f>
+        <v>Framework Orchestrator</v>
+      </c>
+      <c r="D397" s="5" t="str">
+        <f t="array" ref="D397">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A396)-1, 23)+1, INT((ROW(A396)-1)/23)+1)</f>
+        <v>explicit</v>
+      </c>
+      <c r="E397" s="10" t="s">
+        <v>542</v>
+      </c>
+      <c r="F397" s="11" t="s">
+        <v>543</v>
+      </c>
+      <c r="G397" s="11" t="s">
+        <v>544</v>
+      </c>
       <c r="H397" s="9"/>
       <c r="I397" s="9"/>
       <c r="J397" s="9"/>
@@ -49701,13 +51667,31 @@
       <c r="Z397" s="9"/>
     </row>
     <row r="398">
-      <c r="A398" s="9"/>
-      <c r="B398" s="9"/>
-      <c r="C398" s="9"/>
-      <c r="D398" s="9"/>
-      <c r="E398" s="9"/>
-      <c r="F398" s="9"/>
-      <c r="G398" s="9"/>
+      <c r="A398" s="5" t="str">
+        <f t="array" ref="A398">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A397)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B398" s="5" t="str">
+        <f t="array" ref="B398">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B397)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C398" s="5" t="str">
+        <f t="array" ref="C398">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A397)-1, 23)+1)</f>
+        <v>Lifecycle Manager</v>
+      </c>
+      <c r="D398" s="5" t="str">
+        <f t="array" ref="D398">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A397)-1, 23)+1, INT((ROW(A397)-1)/23)+1)</f>
+        <v>implicit</v>
+      </c>
+      <c r="E398" s="10" t="s">
+        <v>545</v>
+      </c>
+      <c r="F398" s="11" t="s">
+        <v>546</v>
+      </c>
+      <c r="G398" s="11" t="s">
+        <v>547</v>
+      </c>
       <c r="H398" s="9"/>
       <c r="I398" s="9"/>
       <c r="J398" s="9"/>
@@ -49729,12 +51713,28 @@
       <c r="Z398" s="9"/>
     </row>
     <row r="399">
-      <c r="A399" s="9"/>
-      <c r="B399" s="9"/>
-      <c r="C399" s="9"/>
-      <c r="D399" s="9"/>
-      <c r="E399" s="9"/>
-      <c r="F399" s="9"/>
+      <c r="A399" s="5" t="str">
+        <f t="array" ref="A399">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A398)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B399" s="5" t="str">
+        <f t="array" ref="B399">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B398)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C399" s="5" t="str">
+        <f t="array" ref="C399">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A398)-1, 23)+1)</f>
+        <v>Configuration Manager</v>
+      </c>
+      <c r="D399" s="5" t="str">
+        <f t="array" ref="D399">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A398)-1, 23)+1, INT((ROW(A398)-1)/23)+1)</f>
+        <v>explicit</v>
+      </c>
+      <c r="E399" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="F399" s="11" t="s">
+        <v>549</v>
+      </c>
       <c r="G399" s="9"/>
       <c r="H399" s="9"/>
       <c r="I399" s="9"/>
@@ -49757,13 +51757,31 @@
       <c r="Z399" s="9"/>
     </row>
     <row r="400">
-      <c r="A400" s="9"/>
-      <c r="B400" s="9"/>
-      <c r="C400" s="9"/>
-      <c r="D400" s="9"/>
-      <c r="E400" s="9"/>
-      <c r="F400" s="9"/>
-      <c r="G400" s="9"/>
+      <c r="A400" s="5" t="str">
+        <f t="array" ref="A400">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A399)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B400" s="5" t="str">
+        <f t="array" ref="B400">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B399)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C400" s="5" t="str">
+        <f t="array" ref="C400">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A399)-1, 23)+1)</f>
+        <v>Multi-Agent Coordinator</v>
+      </c>
+      <c r="D400" s="5" t="str">
+        <f t="array" ref="D400">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A399)-1, 23)+1, INT((ROW(A399)-1)/23)+1)</f>
+        <v>implicit</v>
+      </c>
+      <c r="E400" s="15" t="s">
+        <v>550</v>
+      </c>
+      <c r="F400" s="11" t="s">
+        <v>551</v>
+      </c>
+      <c r="G400" s="11" t="s">
+        <v>552</v>
+      </c>
       <c r="H400" s="9"/>
       <c r="I400" s="9"/>
       <c r="J400" s="9"/>
@@ -49785,10 +51803,23 @@
       <c r="Z400" s="9"/>
     </row>
     <row r="401">
-      <c r="A401" s="9"/>
-      <c r="B401" s="9"/>
-      <c r="C401" s="9"/>
-      <c r="D401" s="9"/>
+      <c r="A401" s="5" t="str">
+        <f t="array" ref="A401">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A400)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B401" s="5" t="str">
+        <f t="array" ref="B401">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B400)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C401" s="5" t="str">
+        <f t="array" ref="C401">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A400)-1, 23)+1)</f>
+        <v>Distributed Execution 
+Coordinator</v>
+      </c>
+      <c r="D401" s="5" t="str">
+        <f t="array" ref="D401">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A400)-1, 23)+1, INT((ROW(A400)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E401" s="9"/>
       <c r="F401" s="9"/>
       <c r="G401" s="9"/>
@@ -49813,13 +51844,31 @@
       <c r="Z401" s="9"/>
     </row>
     <row r="402">
-      <c r="A402" s="9"/>
-      <c r="B402" s="9"/>
-      <c r="C402" s="9"/>
-      <c r="D402" s="9"/>
-      <c r="E402" s="9"/>
-      <c r="F402" s="9"/>
-      <c r="G402" s="9"/>
+      <c r="A402" s="5" t="str">
+        <f t="array" ref="A402">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A401)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B402" s="5" t="str">
+        <f t="array" ref="B402">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B401)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C402" s="5" t="str">
+        <f t="array" ref="C402">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A401)-1, 23)+1)</f>
+        <v>Agent</v>
+      </c>
+      <c r="D402" s="5" t="str">
+        <f t="array" ref="D402">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A401)-1, 23)+1, INT((ROW(A401)-1)/23)+1)</f>
+        <v>explicit</v>
+      </c>
+      <c r="E402" s="10" t="s">
+        <v>553</v>
+      </c>
+      <c r="F402" s="11" t="s">
+        <v>554</v>
+      </c>
+      <c r="G402" s="11" t="s">
+        <v>555</v>
+      </c>
       <c r="H402" s="9"/>
       <c r="I402" s="9"/>
       <c r="J402" s="9"/>
@@ -49841,12 +51890,28 @@
       <c r="Z402" s="9"/>
     </row>
     <row r="403">
-      <c r="A403" s="9"/>
-      <c r="B403" s="9"/>
-      <c r="C403" s="9"/>
-      <c r="D403" s="9"/>
-      <c r="E403" s="9"/>
-      <c r="F403" s="9"/>
+      <c r="A403" s="5" t="str">
+        <f t="array" ref="A403">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A402)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B403" s="5" t="str">
+        <f t="array" ref="B403">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B402)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C403" s="5" t="str">
+        <f t="array" ref="C403">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A402)-1, 23)+1)</f>
+        <v>Function Approximator</v>
+      </c>
+      <c r="D403" s="5" t="str">
+        <f t="array" ref="D403">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A402)-1, 23)+1, INT((ROW(A402)-1)/23)+1)</f>
+        <v>explicit</v>
+      </c>
+      <c r="E403" s="10" t="s">
+        <v>556</v>
+      </c>
+      <c r="F403" s="11" t="s">
+        <v>557</v>
+      </c>
       <c r="G403" s="9"/>
       <c r="H403" s="9"/>
       <c r="I403" s="9"/>
@@ -49869,12 +51934,28 @@
       <c r="Z403" s="9"/>
     </row>
     <row r="404">
-      <c r="A404" s="9"/>
-      <c r="B404" s="9"/>
-      <c r="C404" s="9"/>
-      <c r="D404" s="9"/>
-      <c r="E404" s="9"/>
-      <c r="F404" s="9"/>
+      <c r="A404" s="5" t="str">
+        <f t="array" ref="A404">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A403)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B404" s="5" t="str">
+        <f t="array" ref="B404">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B403)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C404" s="5" t="str">
+        <f t="array" ref="C404">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A403)-1, 23)+1)</f>
+        <v>Buffer</v>
+      </c>
+      <c r="D404" s="5" t="str">
+        <f t="array" ref="D404">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A403)-1, 23)+1, INT((ROW(A403)-1)/23)+1)</f>
+        <v>explicit</v>
+      </c>
+      <c r="E404" s="10" t="s">
+        <v>558</v>
+      </c>
+      <c r="F404" s="11" t="s">
+        <v>559</v>
+      </c>
       <c r="G404" s="9"/>
       <c r="H404" s="9"/>
       <c r="I404" s="9"/>
@@ -49897,13 +51978,31 @@
       <c r="Z404" s="9"/>
     </row>
     <row r="405">
-      <c r="A405" s="9"/>
-      <c r="B405" s="9"/>
-      <c r="C405" s="9"/>
-      <c r="D405" s="9"/>
-      <c r="E405" s="9"/>
-      <c r="F405" s="9"/>
-      <c r="G405" s="9"/>
+      <c r="A405" s="5" t="str">
+        <f t="array" ref="A405">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A404)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B405" s="5" t="str">
+        <f t="array" ref="B405">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B404)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C405" s="5" t="str">
+        <f t="array" ref="C405">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A404)-1, 23)+1)</f>
+        <v>Learner</v>
+      </c>
+      <c r="D405" s="5" t="str">
+        <f t="array" ref="D405">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A404)-1, 23)+1, INT((ROW(A404)-1)/23)+1)</f>
+        <v>explicit</v>
+      </c>
+      <c r="E405" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="F405" s="11" t="s">
+        <v>561</v>
+      </c>
+      <c r="G405" s="11" t="s">
+        <v>562</v>
+      </c>
       <c r="H405" s="9"/>
       <c r="I405" s="9"/>
       <c r="J405" s="9"/>
@@ -49925,10 +52024,22 @@
       <c r="Z405" s="9"/>
     </row>
     <row r="406">
-      <c r="A406" s="9"/>
-      <c r="B406" s="9"/>
-      <c r="C406" s="9"/>
-      <c r="D406" s="9"/>
+      <c r="A406" s="5" t="str">
+        <f t="array" ref="A406">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A405)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B406" s="5" t="str">
+        <f t="array" ref="B406">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B405)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C406" s="5" t="str">
+        <f t="array" ref="C406">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A405)-1, 23)+1)</f>
+        <v>Environment</v>
+      </c>
+      <c r="D406" s="5" t="str">
+        <f t="array" ref="D406">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A405)-1, 23)+1, INT((ROW(A405)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E406" s="9"/>
       <c r="F406" s="9"/>
       <c r="G406" s="9"/>
@@ -49953,10 +52064,22 @@
       <c r="Z406" s="9"/>
     </row>
     <row r="407">
-      <c r="A407" s="9"/>
-      <c r="B407" s="9"/>
-      <c r="C407" s="9"/>
-      <c r="D407" s="9"/>
+      <c r="A407" s="5" t="str">
+        <f t="array" ref="A407">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A406)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B407" s="5" t="str">
+        <f t="array" ref="B407">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B406)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C407" s="5" t="str">
+        <f t="array" ref="C407">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A406)-1, 23)+1)</f>
+        <v>Environment Core</v>
+      </c>
+      <c r="D407" s="5" t="str">
+        <f t="array" ref="D407">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A406)-1, 23)+1, INT((ROW(A406)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E407" s="9"/>
       <c r="F407" s="9"/>
       <c r="G407" s="9"/>
@@ -49981,10 +52104,22 @@
       <c r="Z407" s="9"/>
     </row>
     <row r="408">
-      <c r="A408" s="9"/>
-      <c r="B408" s="9"/>
-      <c r="C408" s="9"/>
-      <c r="D408" s="9"/>
+      <c r="A408" s="5" t="str">
+        <f t="array" ref="A408">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A407)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B408" s="5" t="str">
+        <f t="array" ref="B408">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B407)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C408" s="5" t="str">
+        <f t="array" ref="C408">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A407)-1, 23)+1)</f>
+        <v>Simulator</v>
+      </c>
+      <c r="D408" s="5" t="str">
+        <f t="array" ref="D408">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A407)-1, 23)+1, INT((ROW(A407)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E408" s="9"/>
       <c r="F408" s="9"/>
       <c r="G408" s="9"/>
@@ -50009,10 +52144,22 @@
       <c r="Z408" s="9"/>
     </row>
     <row r="409">
-      <c r="A409" s="9"/>
-      <c r="B409" s="9"/>
-      <c r="C409" s="9"/>
-      <c r="D409" s="9"/>
+      <c r="A409" s="5" t="str">
+        <f t="array" ref="A409">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A408)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B409" s="5" t="str">
+        <f t="array" ref="B409">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B408)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C409" s="5" t="str">
+        <f t="array" ref="C409">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A408)-1, 23)+1)</f>
+        <v>Simulator Adapter</v>
+      </c>
+      <c r="D409" s="5" t="str">
+        <f t="array" ref="D409">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A408)-1, 23)+1, INT((ROW(A408)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E409" s="9"/>
       <c r="F409" s="9"/>
       <c r="G409" s="9"/>
@@ -50037,12 +52184,28 @@
       <c r="Z409" s="9"/>
     </row>
     <row r="410">
-      <c r="A410" s="9"/>
-      <c r="B410" s="9"/>
-      <c r="C410" s="9"/>
-      <c r="D410" s="9"/>
-      <c r="E410" s="9"/>
-      <c r="F410" s="9"/>
+      <c r="A410" s="5" t="str">
+        <f t="array" ref="A410">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A409)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B410" s="5" t="str">
+        <f t="array" ref="B410">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B409)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C410" s="5" t="str">
+        <f t="array" ref="C410">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A409)-1, 23)+1)</f>
+        <v>Checkpoint Manager</v>
+      </c>
+      <c r="D410" s="5" t="str">
+        <f t="array" ref="D410">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A409)-1, 23)+1, INT((ROW(A409)-1)/23)+1)</f>
+        <v>explicit</v>
+      </c>
+      <c r="E410" s="10" t="s">
+        <v>563</v>
+      </c>
+      <c r="F410" s="11" t="s">
+        <v>564</v>
+      </c>
       <c r="G410" s="9"/>
       <c r="H410" s="9"/>
       <c r="I410" s="9"/>
@@ -50065,10 +52228,23 @@
       <c r="Z410" s="9"/>
     </row>
     <row r="411">
-      <c r="A411" s="9"/>
-      <c r="B411" s="9"/>
-      <c r="C411" s="9"/>
-      <c r="D411" s="9"/>
+      <c r="A411" s="5" t="str">
+        <f t="array" ref="A411">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A410)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B411" s="5" t="str">
+        <f t="array" ref="B411">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B410)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C411" s="5" t="str">
+        <f t="array" ref="C411">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A410)-1, 23)+1)</f>
+        <v>Environment Parameter 
+Manager</v>
+      </c>
+      <c r="D411" s="5" t="str">
+        <f t="array" ref="D411">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A410)-1, 23)+1, INT((ROW(A410)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E411" s="9"/>
       <c r="F411" s="9"/>
       <c r="G411" s="9"/>
@@ -50093,10 +52269,22 @@
       <c r="Z411" s="9"/>
     </row>
     <row r="412">
-      <c r="A412" s="9"/>
-      <c r="B412" s="9"/>
-      <c r="C412" s="9"/>
-      <c r="D412" s="9"/>
+      <c r="A412" s="5" t="str">
+        <f t="array" ref="A412">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A411)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B412" s="5" t="str">
+        <f t="array" ref="B412">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B411)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C412" s="5" t="str">
+        <f t="array" ref="C412">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A411)-1, 23)+1)</f>
+        <v>Renderer</v>
+      </c>
+      <c r="D412" s="5" t="str">
+        <f t="array" ref="D412">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A411)-1, 23)+1, INT((ROW(A411)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E412" s="9"/>
       <c r="F412" s="9"/>
       <c r="G412" s="9"/>
@@ -50121,10 +52309,22 @@
       <c r="Z412" s="9"/>
     </row>
     <row r="413">
-      <c r="A413" s="9"/>
-      <c r="B413" s="9"/>
-      <c r="C413" s="9"/>
-      <c r="D413" s="9"/>
+      <c r="A413" s="5" t="str">
+        <f t="array" ref="A413">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A412)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B413" s="5" t="str">
+        <f t="array" ref="B413">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B412)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C413" s="5" t="str">
+        <f t="array" ref="C413">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A412)-1, 23)+1)</f>
+        <v>Recorder</v>
+      </c>
+      <c r="D413" s="5" t="str">
+        <f t="array" ref="D413">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A412)-1, 23)+1, INT((ROW(A412)-1)/23)+1)</f>
+        <v>not implemented</v>
+      </c>
       <c r="E413" s="9"/>
       <c r="F413" s="9"/>
       <c r="G413" s="9"/>
@@ -50149,14 +52349,34 @@
       <c r="Z413" s="9"/>
     </row>
     <row r="414">
-      <c r="A414" s="9"/>
-      <c r="B414" s="9"/>
-      <c r="C414" s="9"/>
-      <c r="D414" s="9"/>
-      <c r="E414" s="9"/>
-      <c r="F414" s="9"/>
-      <c r="G414" s="9"/>
-      <c r="H414" s="9"/>
+      <c r="A414" s="5" t="str">
+        <f t="array" ref="A414">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A413)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B414" s="5" t="str">
+        <f t="array" ref="B414">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B413)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C414" s="5" t="str">
+        <f t="array" ref="C414">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A413)-1, 23)+1)</f>
+        <v>Logger</v>
+      </c>
+      <c r="D414" s="5" t="str">
+        <f t="array" ref="D414">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A413)-1, 23)+1, INT((ROW(A413)-1)/23)+1)</f>
+        <v>external</v>
+      </c>
+      <c r="E414" s="10" t="s">
+        <v>565</v>
+      </c>
+      <c r="F414" s="11" t="s">
+        <v>566</v>
+      </c>
+      <c r="G414" s="11" t="s">
+        <v>567</v>
+      </c>
+      <c r="H414" s="11" t="s">
+        <v>568</v>
+      </c>
       <c r="I414" s="9"/>
       <c r="J414" s="9"/>
       <c r="K414" s="9"/>
@@ -50177,14 +52397,34 @@
       <c r="Z414" s="9"/>
     </row>
     <row r="415">
-      <c r="A415" s="9"/>
-      <c r="B415" s="9"/>
-      <c r="C415" s="9"/>
-      <c r="D415" s="9"/>
-      <c r="E415" s="9"/>
-      <c r="F415" s="9"/>
-      <c r="G415" s="9"/>
-      <c r="H415" s="9"/>
+      <c r="A415" s="5" t="str">
+        <f t="array" ref="A415">INDEX('final-RA-to-framework-summary'!$C$1:$T$1, 1, INT((ROW(A414)-1)/23)+1)</f>
+        <v>F18</v>
+      </c>
+      <c r="B415" s="5" t="str">
+        <f t="array" ref="B415">INDEX('final-RA-to-framework-summary'!$C$2:$T$2, 1, INT((ROW(B414)-1)/23)+1)</f>
+        <v>Tianshou</v>
+      </c>
+      <c r="C415" s="5" t="str">
+        <f t="array" ref="C415">INDEX('final-RA-to-framework-summary'!$B$4:$B$26, MOD(ROW(A414)-1, 23)+1)</f>
+        <v>Reporter</v>
+      </c>
+      <c r="D415" s="5" t="str">
+        <f t="array" ref="D415">INDEX('final-RA-to-framework-summary'!$C$4:$Z$26, MOD(ROW(A414)-1, 23)+1, INT((ROW(A414)-1)/23)+1)</f>
+        <v>external</v>
+      </c>
+      <c r="E415" s="15" t="s">
+        <v>569</v>
+      </c>
+      <c r="F415" s="11" t="s">
+        <v>566</v>
+      </c>
+      <c r="G415" s="11" t="s">
+        <v>570</v>
+      </c>
+      <c r="H415" s="11" t="s">
+        <v>571</v>
+      </c>
       <c r="I415" s="9"/>
       <c r="J415" s="9"/>
       <c r="K415" s="9"/>
@@ -66747,44 +68987,95 @@
     <hyperlink r:id="rId103" ref="E253"/>
     <hyperlink r:id="rId104" ref="E254"/>
     <hyperlink r:id="rId105" ref="E256"/>
-    <hyperlink r:id="rId106" ref="E259"/>
-    <hyperlink r:id="rId107" ref="E260"/>
-    <hyperlink r:id="rId108" ref="E261"/>
-    <hyperlink r:id="rId109" ref="E262"/>
-    <hyperlink r:id="rId110" ref="E263"/>
-    <hyperlink r:id="rId111" ref="E264"/>
-    <hyperlink r:id="rId112" ref="E265"/>
-    <hyperlink r:id="rId113" ref="E266"/>
-    <hyperlink r:id="rId114" ref="E267"/>
-    <hyperlink r:id="rId115" ref="E272"/>
-    <hyperlink r:id="rId116" ref="E273"/>
-    <hyperlink r:id="rId117" ref="E277"/>
-    <hyperlink r:id="rId118" ref="E279"/>
-    <hyperlink r:id="rId119" ref="E282"/>
-    <hyperlink r:id="rId120" ref="E283"/>
-    <hyperlink r:id="rId121" ref="E286"/>
-    <hyperlink r:id="rId122" ref="E287"/>
-    <hyperlink r:id="rId123" ref="E288"/>
-    <hyperlink r:id="rId124" ref="E289"/>
-    <hyperlink r:id="rId125" ref="E290"/>
-    <hyperlink r:id="rId126" ref="E295"/>
-    <hyperlink r:id="rId127" ref="E298"/>
-    <hyperlink r:id="rId128" ref="E299"/>
-    <hyperlink r:id="rId129" ref="E302"/>
-    <hyperlink r:id="rId130" ref="E303"/>
-    <hyperlink r:id="rId131" ref="E305"/>
-    <hyperlink r:id="rId132" ref="E306"/>
-    <hyperlink r:id="rId133" ref="E307"/>
-    <hyperlink r:id="rId134" ref="E308"/>
-    <hyperlink r:id="rId135" ref="E309"/>
-    <hyperlink r:id="rId136" ref="E310"/>
-    <hyperlink r:id="rId137" ref="E311"/>
-    <hyperlink r:id="rId138" ref="E312"/>
-    <hyperlink r:id="rId139" ref="E313"/>
-    <hyperlink r:id="rId140" ref="E318"/>
-    <hyperlink r:id="rId141" ref="E322"/>
-    <hyperlink r:id="rId142" ref="E323"/>
+    <hyperlink r:id="rId106" ref="E257"/>
+    <hyperlink r:id="rId107" ref="E259"/>
+    <hyperlink r:id="rId108" ref="E260"/>
+    <hyperlink r:id="rId109" ref="E261"/>
+    <hyperlink r:id="rId110" ref="E262"/>
+    <hyperlink r:id="rId111" ref="E263"/>
+    <hyperlink r:id="rId112" ref="E264"/>
+    <hyperlink r:id="rId113" ref="E265"/>
+    <hyperlink r:id="rId114" ref="E266"/>
+    <hyperlink r:id="rId115" ref="E267"/>
+    <hyperlink r:id="rId116" ref="E272"/>
+    <hyperlink r:id="rId117" ref="E273"/>
+    <hyperlink r:id="rId118" ref="E277"/>
+    <hyperlink r:id="rId119" ref="E279"/>
+    <hyperlink r:id="rId120" ref="E282"/>
+    <hyperlink r:id="rId121" ref="E283"/>
+    <hyperlink r:id="rId122" ref="E286"/>
+    <hyperlink r:id="rId123" ref="E287"/>
+    <hyperlink r:id="rId124" ref="E288"/>
+    <hyperlink r:id="rId125" ref="E289"/>
+    <hyperlink r:id="rId126" ref="E290"/>
+    <hyperlink r:id="rId127" ref="E295"/>
+    <hyperlink r:id="rId128" ref="E298"/>
+    <hyperlink r:id="rId129" ref="E299"/>
+    <hyperlink r:id="rId130" ref="E302"/>
+    <hyperlink r:id="rId131" ref="E303"/>
+    <hyperlink r:id="rId132" ref="E305"/>
+    <hyperlink r:id="rId133" ref="E306"/>
+    <hyperlink r:id="rId134" ref="E307"/>
+    <hyperlink r:id="rId135" ref="E308"/>
+    <hyperlink r:id="rId136" ref="E309"/>
+    <hyperlink r:id="rId137" ref="E310"/>
+    <hyperlink r:id="rId138" ref="E311"/>
+    <hyperlink r:id="rId139" ref="E312"/>
+    <hyperlink r:id="rId140" ref="E313"/>
+    <hyperlink r:id="rId141" ref="E318"/>
+    <hyperlink r:id="rId142" ref="E322"/>
+    <hyperlink r:id="rId143" ref="E323"/>
+    <hyperlink r:id="rId144" ref="E325"/>
+    <hyperlink r:id="rId145" ref="E327"/>
+    <hyperlink r:id="rId146" ref="E328"/>
+    <hyperlink r:id="rId147" ref="E329"/>
+    <hyperlink r:id="rId148" ref="E330"/>
+    <hyperlink r:id="rId149" ref="E331"/>
+    <hyperlink r:id="rId150" ref="E333"/>
+    <hyperlink r:id="rId151" ref="E334"/>
+    <hyperlink r:id="rId152" ref="E335"/>
+    <hyperlink r:id="rId153" ref="E336"/>
+    <hyperlink r:id="rId154" ref="E341"/>
+    <hyperlink r:id="rId155" ref="E344"/>
+    <hyperlink r:id="rId156" ref="E345"/>
+    <hyperlink r:id="rId157" ref="E346"/>
+    <hyperlink r:id="rId158" ref="E348"/>
+    <hyperlink r:id="rId159" ref="E351"/>
+    <hyperlink r:id="rId160" ref="E352"/>
+    <hyperlink r:id="rId161" ref="E353"/>
+    <hyperlink r:id="rId162" ref="E355"/>
+    <hyperlink r:id="rId163" ref="E356"/>
+    <hyperlink r:id="rId164" ref="E357"/>
+    <hyperlink r:id="rId165" ref="E358"/>
+    <hyperlink r:id="rId166" ref="E359"/>
+    <hyperlink r:id="rId167" ref="E364"/>
+    <hyperlink r:id="rId168" ref="E368"/>
+    <hyperlink r:id="rId169" ref="E369"/>
+    <hyperlink r:id="rId170" ref="E371"/>
+    <hyperlink r:id="rId171" ref="E374"/>
+    <hyperlink r:id="rId172" ref="E375"/>
+    <hyperlink r:id="rId173" ref="E376"/>
+    <hyperlink r:id="rId174" ref="E379"/>
+    <hyperlink r:id="rId175" ref="E380"/>
+    <hyperlink r:id="rId176" ref="E381"/>
+    <hyperlink r:id="rId177" ref="E382"/>
+    <hyperlink r:id="rId178" ref="E387"/>
+    <hyperlink r:id="rId179" ref="E390"/>
+    <hyperlink r:id="rId180" ref="E391"/>
+    <hyperlink r:id="rId181" ref="E392"/>
+    <hyperlink r:id="rId182" ref="E394"/>
+    <hyperlink r:id="rId183" ref="E397"/>
+    <hyperlink r:id="rId184" ref="E398"/>
+    <hyperlink r:id="rId185" ref="E399"/>
+    <hyperlink r:id="rId186" ref="E400"/>
+    <hyperlink r:id="rId187" ref="E402"/>
+    <hyperlink r:id="rId188" ref="E403"/>
+    <hyperlink r:id="rId189" ref="E404"/>
+    <hyperlink r:id="rId190" ref="E405"/>
+    <hyperlink r:id="rId191" ref="E410"/>
+    <hyperlink r:id="rId192" ref="E414"/>
+    <hyperlink r:id="rId193" ref="E415"/>
   </hyperlinks>
-  <drawing r:id="rId143"/>
+  <drawing r:id="rId194"/>
 </worksheet>
 </file>
</xml_diff>